<commit_message>
Buildings and Transportation updates (transport involved reallocation of certain vehicle types)
</commit_message>
<xml_diff>
--- a/InputData/trans/AVL/Avg Vehicle Lifetime.xlsx
+++ b/InputData/trans/AVL/Avg Vehicle Lifetime.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rachel Goldstein\Desktop\EPS Models\SouthKorea EPS\InputData\trans\AVL\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\administer\Dropbox\kjh\2026\01.EPS\01.EI\01.메일\260108_메일회신\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EF34157-7591-4A0D-850C-5B993E103A87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1944F64F-AD81-4996-A4B5-75E70CAE79BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="32595" yWindow="3795" windowWidth="20145" windowHeight="11235" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="9" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="132">
   <si>
     <t>Car Avg Lifetime, years (Page 22, Table 7)</t>
   </si>
@@ -463,27 +463,39 @@
     <t>Source: Decommissioning cycles by year (https://v.daum.net/v/E5WSO03fTV)</t>
     <phoneticPr fontId="38" type="noConversion"/>
   </si>
+  <si>
+    <t>Passenger</t>
+    <phoneticPr fontId="38" type="noConversion"/>
+  </si>
+  <si>
+    <t>LDV+HDV</t>
+    <phoneticPr fontId="38" type="noConversion"/>
+  </si>
+  <si>
+    <t>freight</t>
+    <phoneticPr fontId="38" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
   <numFmts count="9">
-    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="164" formatCode="###0.00_)"/>
-    <numFmt numFmtId="165" formatCode="\(\R\)General"/>
-    <numFmt numFmtId="166" formatCode="\(\R\)\ ###0"/>
-    <numFmt numFmtId="167" formatCode="0.0"/>
-    <numFmt numFmtId="168" formatCode="\(\R\)0.0"/>
-    <numFmt numFmtId="169" formatCode="#,##0_)"/>
-    <numFmt numFmtId="170" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="171" formatCode="_(* #,##0.0_);_(* \(#,##0.0\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="176" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="177" formatCode="###0.00_)"/>
+    <numFmt numFmtId="178" formatCode="\(\R\)General"/>
+    <numFmt numFmtId="179" formatCode="\(\R\)\ ###0"/>
+    <numFmt numFmtId="180" formatCode="0.0"/>
+    <numFmt numFmtId="181" formatCode="\(\R\)0.0"/>
+    <numFmt numFmtId="182" formatCode="#,##0_)"/>
+    <numFmt numFmtId="183" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="184" formatCode="_(* #,##0.0_);_(* \(#,##0.0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="40">
+  <fonts count="40" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="맑은 고딕"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -491,7 +503,7 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="맑은 고딕"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -499,7 +511,7 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
-      <name val="Calibri"/>
+      <name val="맑은 고딕"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -507,14 +519,14 @@
       <b/>
       <sz val="9"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="맑은 고딕"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="9"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="맑은 고딕"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -522,7 +534,7 @@
       <u/>
       <sz val="10"/>
       <color theme="4"/>
-      <name val="Calibri"/>
+      <name val="맑은 고딕"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -537,7 +549,7 @@
       <b/>
       <sz val="12"/>
       <color theme="4"/>
-      <name val="Calibri"/>
+      <name val="맑은 고딕"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -554,14 +566,14 @@
       <i/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="맑은 고딕"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="맑은 고딕"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -569,7 +581,7 @@
       <b/>
       <sz val="18"/>
       <color theme="3"/>
-      <name val="Cambria"/>
+      <name val="맑은 고딕"/>
       <family val="2"/>
       <scheme val="major"/>
     </font>
@@ -577,7 +589,7 @@
       <b/>
       <sz val="15"/>
       <color theme="3"/>
-      <name val="Calibri"/>
+      <name val="맑은 고딕"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -585,7 +597,7 @@
       <b/>
       <sz val="13"/>
       <color theme="3"/>
-      <name val="Calibri"/>
+      <name val="맑은 고딕"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -593,35 +605,35 @@
       <b/>
       <sz val="11"/>
       <color theme="3"/>
-      <name val="Calibri"/>
+      <name val="맑은 고딕"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF006100"/>
-      <name val="Calibri"/>
+      <name val="맑은 고딕"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
+      <name val="맑은 고딕"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF9C6500"/>
-      <name val="Calibri"/>
+      <name val="맑은 고딕"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF3F3F76"/>
-      <name val="Calibri"/>
+      <name val="맑은 고딕"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -629,7 +641,7 @@
       <b/>
       <sz val="11"/>
       <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
+      <name val="맑은 고딕"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -637,14 +649,14 @@
       <b/>
       <sz val="11"/>
       <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
+      <name val="맑은 고딕"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
+      <name val="맑은 고딕"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -652,14 +664,14 @@
       <b/>
       <sz val="11"/>
       <color theme="0"/>
-      <name val="Calibri"/>
+      <name val="맑은 고딕"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
+      <name val="맑은 고딕"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -667,21 +679,21 @@
       <i/>
       <sz val="11"/>
       <color rgb="FF7F7F7F"/>
-      <name val="Calibri"/>
+      <name val="맑은 고딕"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="0"/>
-      <name val="Calibri"/>
+      <name val="맑은 고딕"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
-      <name val="Calibri"/>
+      <name val="맑은 고딕"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -738,13 +750,13 @@
       <i/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="맑은 고딕"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="8"/>
-      <name val="Calibri"/>
+      <name val="맑은 고딕"/>
       <family val="3"/>
       <charset val="129"/>
       <scheme val="minor"/>
@@ -752,7 +764,7 @@
     <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
+      <name val="맑은 고딕"/>
       <family val="3"/>
       <charset val="129"/>
       <scheme val="minor"/>
@@ -1330,7 +1342,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyProtection="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0">
+    <xf numFmtId="177" fontId="8" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="10">
@@ -1387,10 +1399,10 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="10">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="33" fillId="0" borderId="10">
+    <xf numFmtId="182" fontId="33" fillId="0" borderId="10">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="43" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="176" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="85">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -1495,10 +1507,10 @@
     <xf numFmtId="1" fontId="30" fillId="0" borderId="29" xfId="59" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="30" fillId="0" borderId="29" xfId="59" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="178" fontId="30" fillId="0" borderId="29" xfId="59" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="30" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="178" fontId="30" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="29" xfId="59" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1510,7 +1522,7 @@
     <xf numFmtId="1" fontId="30" fillId="0" borderId="0" xfId="59" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="30" fillId="0" borderId="0" xfId="59" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="179" fontId="30" fillId="0" borderId="0" xfId="59" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1530,21 +1542,21 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="3" fontId="31" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="167" fontId="30" fillId="0" borderId="0" xfId="60" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="180" fontId="30" fillId="0" borderId="0" xfId="60" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="167" fontId="31" fillId="0" borderId="0" xfId="16" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="167" fontId="31" fillId="0" borderId="0" xfId="16" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="31" fillId="0" borderId="0" xfId="16" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="180" fontId="31" fillId="0" borderId="0" xfId="16" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="180" fontId="31" fillId="0" borderId="0" xfId="16" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="181" fontId="31" fillId="0" borderId="0" xfId="16" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="3" fontId="31" fillId="0" borderId="0" xfId="61" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="167" fontId="31" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="180" fontId="31" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="31" fillId="0" borderId="27" xfId="60" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
     </xf>
-    <xf numFmtId="167" fontId="31" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="180" fontId="31" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="31" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1567,16 +1579,25 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="62" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="170" fontId="37" fillId="0" borderId="0" xfId="62" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="183" fontId="0" fillId="0" borderId="0" xfId="62" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="183" fontId="37" fillId="0" borderId="0" xfId="62" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="9" fontId="0" fillId="36" borderId="0" xfId="16" applyFont="1" applyFill="1"/>
     <xf numFmtId="1" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="170" fontId="24" fillId="0" borderId="0" xfId="62" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="170" fontId="39" fillId="0" borderId="0" xfId="62" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="171" fontId="39" fillId="0" borderId="0" xfId="62" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="183" fontId="24" fillId="0" borderId="0" xfId="62" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="183" fontId="39" fillId="0" borderId="0" xfId="62" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="184" fontId="39" fillId="0" borderId="0" xfId="62" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="35" fillId="0" borderId="0" xfId="15" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="27" xfId="58" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -1589,80 +1610,71 @@
     <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="15" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="63">
-    <cellStyle name="20% - Accent1" xfId="35" builtinId="30" customBuiltin="1"/>
-    <cellStyle name="20% - Accent2" xfId="39" builtinId="34" customBuiltin="1"/>
-    <cellStyle name="20% - Accent3" xfId="43" builtinId="38" customBuiltin="1"/>
-    <cellStyle name="20% - Accent4" xfId="47" builtinId="42" customBuiltin="1"/>
-    <cellStyle name="20% - Accent5" xfId="51" builtinId="46" customBuiltin="1"/>
-    <cellStyle name="20% - Accent6" xfId="55" builtinId="50" customBuiltin="1"/>
-    <cellStyle name="40% - Accent1" xfId="36" builtinId="31" customBuiltin="1"/>
-    <cellStyle name="40% - Accent2" xfId="40" builtinId="35" customBuiltin="1"/>
-    <cellStyle name="40% - Accent3" xfId="44" builtinId="39" customBuiltin="1"/>
-    <cellStyle name="40% - Accent4" xfId="48" builtinId="43" customBuiltin="1"/>
-    <cellStyle name="40% - Accent5" xfId="52" builtinId="47" customBuiltin="1"/>
-    <cellStyle name="40% - Accent6" xfId="56" builtinId="51" customBuiltin="1"/>
-    <cellStyle name="60% - Accent1" xfId="37" builtinId="32" customBuiltin="1"/>
-    <cellStyle name="60% - Accent2" xfId="41" builtinId="36" customBuiltin="1"/>
-    <cellStyle name="60% - Accent3" xfId="45" builtinId="40" customBuiltin="1"/>
-    <cellStyle name="60% - Accent4" xfId="49" builtinId="44" customBuiltin="1"/>
-    <cellStyle name="60% - Accent5" xfId="53" builtinId="48" customBuiltin="1"/>
-    <cellStyle name="60% - Accent6" xfId="57" builtinId="52" customBuiltin="1"/>
-    <cellStyle name="Accent1" xfId="34" builtinId="29" customBuiltin="1"/>
-    <cellStyle name="Accent2" xfId="38" builtinId="33" customBuiltin="1"/>
-    <cellStyle name="Accent3" xfId="42" builtinId="37" customBuiltin="1"/>
-    <cellStyle name="Accent4" xfId="46" builtinId="41" customBuiltin="1"/>
-    <cellStyle name="Accent5" xfId="50" builtinId="45" customBuiltin="1"/>
-    <cellStyle name="Accent6" xfId="54" builtinId="49" customBuiltin="1"/>
-    <cellStyle name="Bad" xfId="23" builtinId="27" customBuiltin="1"/>
+    <cellStyle name="20% - 강조색1" xfId="35" builtinId="30" customBuiltin="1"/>
+    <cellStyle name="20% - 강조색2" xfId="39" builtinId="34" customBuiltin="1"/>
+    <cellStyle name="20% - 강조색3" xfId="43" builtinId="38" customBuiltin="1"/>
+    <cellStyle name="20% - 강조색4" xfId="47" builtinId="42" customBuiltin="1"/>
+    <cellStyle name="20% - 강조색5" xfId="51" builtinId="46" customBuiltin="1"/>
+    <cellStyle name="20% - 강조색6" xfId="55" builtinId="50" customBuiltin="1"/>
+    <cellStyle name="40% - 강조색1" xfId="36" builtinId="31" customBuiltin="1"/>
+    <cellStyle name="40% - 강조색2" xfId="40" builtinId="35" customBuiltin="1"/>
+    <cellStyle name="40% - 강조색3" xfId="44" builtinId="39" customBuiltin="1"/>
+    <cellStyle name="40% - 강조색4" xfId="48" builtinId="43" customBuiltin="1"/>
+    <cellStyle name="40% - 강조색5" xfId="52" builtinId="47" customBuiltin="1"/>
+    <cellStyle name="40% - 강조색6" xfId="56" builtinId="51" customBuiltin="1"/>
+    <cellStyle name="60% - 강조색1" xfId="37" builtinId="32" customBuiltin="1"/>
+    <cellStyle name="60% - 강조색2" xfId="41" builtinId="36" customBuiltin="1"/>
+    <cellStyle name="60% - 강조색3" xfId="45" builtinId="40" customBuiltin="1"/>
+    <cellStyle name="60% - 강조색4" xfId="49" builtinId="44" customBuiltin="1"/>
+    <cellStyle name="60% - 강조색5" xfId="53" builtinId="48" customBuiltin="1"/>
+    <cellStyle name="60% - 강조색6" xfId="57" builtinId="52" customBuiltin="1"/>
     <cellStyle name="Body: normal cell" xfId="3" xr:uid="{00000000-0005-0000-0000-000019000000}"/>
-    <cellStyle name="Calculation" xfId="27" builtinId="22" customBuiltin="1"/>
-    <cellStyle name="Check Cell" xfId="29" builtinId="23" customBuiltin="1"/>
-    <cellStyle name="Comma" xfId="62" builtinId="3"/>
     <cellStyle name="Data" xfId="14" xr:uid="{00000000-0005-0000-0000-00001C000000}"/>
     <cellStyle name="Data no deci" xfId="61" xr:uid="{00000000-0005-0000-0000-00001D000000}"/>
-    <cellStyle name="Explanatory Text" xfId="32" builtinId="53" customBuiltin="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="11" builtinId="9" customBuiltin="1"/>
     <cellStyle name="Font: Calibri, 9pt regular" xfId="9" xr:uid="{00000000-0005-0000-0000-000020000000}"/>
     <cellStyle name="Footnotes: all except top row" xfId="12" xr:uid="{00000000-0005-0000-0000-000021000000}"/>
     <cellStyle name="Footnotes: top row" xfId="7" xr:uid="{00000000-0005-0000-0000-000022000000}"/>
-    <cellStyle name="Good" xfId="22" builtinId="26" customBuiltin="1"/>
     <cellStyle name="Header: bottom row" xfId="2" xr:uid="{00000000-0005-0000-0000-000024000000}"/>
     <cellStyle name="Header: top rows" xfId="4" xr:uid="{00000000-0005-0000-0000-000025000000}"/>
-    <cellStyle name="Heading 1" xfId="18" builtinId="16" customBuiltin="1"/>
-    <cellStyle name="Heading 2" xfId="19" builtinId="17" customBuiltin="1"/>
-    <cellStyle name="Heading 3" xfId="20" builtinId="18" customBuiltin="1"/>
-    <cellStyle name="Heading 4" xfId="21" builtinId="19" customBuiltin="1"/>
     <cellStyle name="Hed Side" xfId="15" xr:uid="{00000000-0005-0000-0000-00002A000000}"/>
     <cellStyle name="Hed Side Regular" xfId="60" xr:uid="{00000000-0005-0000-0000-00002B000000}"/>
     <cellStyle name="Hed Top" xfId="59" xr:uid="{00000000-0005-0000-0000-00002C000000}"/>
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Hyperlink 2" xfId="10" xr:uid="{00000000-0005-0000-0000-00002E000000}"/>
-    <cellStyle name="Input" xfId="25" builtinId="20" customBuiltin="1"/>
-    <cellStyle name="Linked Cell" xfId="28" builtinId="24" customBuiltin="1"/>
-    <cellStyle name="Neutral" xfId="24" builtinId="28" customBuiltin="1"/>
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Note" xfId="31" builtinId="10" customBuiltin="1"/>
-    <cellStyle name="Output" xfId="26" builtinId="21" customBuiltin="1"/>
     <cellStyle name="Parent row" xfId="6" xr:uid="{00000000-0005-0000-0000-000035000000}"/>
-    <cellStyle name="Percent" xfId="16" builtinId="5"/>
     <cellStyle name="Section Break" xfId="8" xr:uid="{00000000-0005-0000-0000-000037000000}"/>
     <cellStyle name="Section Break: parent row" xfId="5" xr:uid="{00000000-0005-0000-0000-000038000000}"/>
     <cellStyle name="Table title" xfId="13" xr:uid="{00000000-0005-0000-0000-000039000000}"/>
-    <cellStyle name="Title" xfId="17" builtinId="15" customBuiltin="1"/>
     <cellStyle name="Title-2" xfId="58" xr:uid="{00000000-0005-0000-0000-00003B000000}"/>
-    <cellStyle name="Total" xfId="33" builtinId="25" customBuiltin="1"/>
-    <cellStyle name="Warning Text" xfId="30" builtinId="11" customBuiltin="1"/>
+    <cellStyle name="강조색1" xfId="34" builtinId="29" customBuiltin="1"/>
+    <cellStyle name="강조색2" xfId="38" builtinId="33" customBuiltin="1"/>
+    <cellStyle name="강조색3" xfId="42" builtinId="37" customBuiltin="1"/>
+    <cellStyle name="강조색4" xfId="46" builtinId="41" customBuiltin="1"/>
+    <cellStyle name="강조색5" xfId="50" builtinId="45" customBuiltin="1"/>
+    <cellStyle name="강조색6" xfId="54" builtinId="49" customBuiltin="1"/>
+    <cellStyle name="경고문" xfId="30" builtinId="11" customBuiltin="1"/>
+    <cellStyle name="계산" xfId="27" builtinId="22" customBuiltin="1"/>
+    <cellStyle name="나쁨" xfId="23" builtinId="27" customBuiltin="1"/>
+    <cellStyle name="메모" xfId="31" builtinId="10" customBuiltin="1"/>
+    <cellStyle name="백분율" xfId="16" builtinId="5"/>
+    <cellStyle name="보통" xfId="24" builtinId="28" customBuiltin="1"/>
+    <cellStyle name="설명 텍스트" xfId="32" builtinId="53" customBuiltin="1"/>
+    <cellStyle name="셀 확인" xfId="29" builtinId="23" customBuiltin="1"/>
+    <cellStyle name="쉼표" xfId="62" builtinId="3"/>
+    <cellStyle name="연결된 셀" xfId="28" builtinId="24" customBuiltin="1"/>
+    <cellStyle name="열어 본 하이퍼링크" xfId="11" builtinId="9" customBuiltin="1"/>
+    <cellStyle name="요약" xfId="33" builtinId="25" customBuiltin="1"/>
+    <cellStyle name="입력" xfId="25" builtinId="20" customBuiltin="1"/>
+    <cellStyle name="제목" xfId="17" builtinId="15" customBuiltin="1"/>
+    <cellStyle name="제목 1" xfId="18" builtinId="16" customBuiltin="1"/>
+    <cellStyle name="제목 2" xfId="19" builtinId="17" customBuiltin="1"/>
+    <cellStyle name="제목 3" xfId="20" builtinId="18" customBuiltin="1"/>
+    <cellStyle name="제목 4" xfId="21" builtinId="19" customBuiltin="1"/>
+    <cellStyle name="좋음" xfId="22" builtinId="26" customBuiltin="1"/>
+    <cellStyle name="출력" xfId="26" builtinId="21" customBuiltin="1"/>
+    <cellStyle name="표준" xfId="0" builtinId="0"/>
+    <cellStyle name="하이퍼링크" xfId="1" builtinId="8"/>
   </cellStyles>
   <dxfs count="2">
     <dxf>
@@ -1995,17 +2007,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B59"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="132.21875" customWidth="1"/>
+    <col min="2" max="2" width="132.25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>51</v>
       </c>
@@ -2013,233 +2025,232 @@
         <v>53</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B4" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B5" s="9">
         <v>2006</v>
       </c>
     </row>
-    <row r="6" spans="1:2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B6" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B7" s="4" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:2">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B8" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:2">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B10" s="6" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="11" spans="1:2">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B11" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="12" spans="1:2">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B12" s="9">
         <v>2016</v>
       </c>
     </row>
-    <row r="13" spans="1:2">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B13" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="14" spans="1:2">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B14" s="4" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:2">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B15" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="17" spans="2:2">
+    <row r="17" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B17" s="6" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="18" spans="2:2">
+    <row r="18" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B18" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="19" spans="2:2">
+    <row r="19" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B19" s="9">
         <v>2015</v>
       </c>
     </row>
-    <row r="20" spans="2:2">
+    <row r="20" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B20" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="21" spans="2:2">
+    <row r="21" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B21" s="4" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="22" spans="2:2">
+    <row r="22" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B22" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="23" spans="2:2"/>
-    <row r="24" spans="2:2">
+    <row r="24" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B24" s="6" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="25" spans="2:2">
+    <row r="25" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B25" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="26" spans="2:2">
+    <row r="26" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B26" s="9">
         <v>2019</v>
       </c>
     </row>
-    <row r="27" spans="2:2">
+    <row r="27" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B27" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="28" spans="2:2">
+    <row r="28" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B28" s="4" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="30" spans="2:2">
+    <row r="30" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B30" s="6" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="31" spans="2:2">
+    <row r="31" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B31" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="32" spans="2:2">
+    <row r="32" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B32" s="9">
         <v>2013</v>
       </c>
     </row>
-    <row r="33" spans="2:2">
+    <row r="33" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B33" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="34" spans="2:2">
+    <row r="34" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B34" s="4" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="35" spans="2:2">
+    <row r="35" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B35" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="37" spans="2:2">
+    <row r="37" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B37" s="6" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="38" spans="2:2">
+    <row r="38" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B38" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="39" spans="2:2">
+    <row r="39" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B39" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="40" spans="2:2">
+    <row r="40" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B40" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="41" spans="2:2">
+    <row r="41" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B41" s="19" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="42" spans="2:2">
+    <row r="42" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B42" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="44" spans="2:2">
+    <row r="44" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B44" s="6" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="45" spans="2:2">
+    <row r="45" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B45" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="46" spans="2:2">
+    <row r="46" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B46" s="9">
         <v>2009</v>
       </c>
     </row>
-    <row r="47" spans="2:2">
+    <row r="47" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B47" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="48" spans="2:2">
+    <row r="48" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B48" s="19" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="49" spans="1:2">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B49" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="51" spans="1:2">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A51" s="1" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="52" spans="1:2">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="54" spans="1:2">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="55" spans="1:2">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="57" spans="1:2">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="59" spans="1:2">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>99</v>
       </c>
@@ -2260,72 +2271,72 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:BB61"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="9.125" defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="19.33203125" customWidth="1"/>
-    <col min="2" max="27" width="7.77734375" customWidth="1"/>
-    <col min="28" max="28" width="7.109375" customWidth="1"/>
+    <col min="1" max="1" width="19.375" customWidth="1"/>
+    <col min="2" max="27" width="7.75" customWidth="1"/>
+    <col min="28" max="28" width="7.125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:54" ht="16.5" customHeight="1" thickBot="1">
-      <c r="A1" s="78" t="s">
+    <row r="1" spans="1:54" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="81" t="s">
         <v>64</v>
       </c>
-      <c r="B1" s="78"/>
-      <c r="C1" s="78"/>
-      <c r="D1" s="78"/>
-      <c r="E1" s="78"/>
-      <c r="F1" s="78"/>
-      <c r="G1" s="78"/>
-      <c r="H1" s="78"/>
-      <c r="I1" s="78"/>
-      <c r="J1" s="78"/>
-      <c r="K1" s="78"/>
-      <c r="L1" s="78"/>
-      <c r="M1" s="78"/>
-      <c r="N1" s="78"/>
-      <c r="O1" s="78"/>
-      <c r="P1" s="78"/>
-      <c r="Q1" s="78"/>
-      <c r="R1" s="78"/>
-      <c r="S1" s="78"/>
-      <c r="T1" s="78"/>
-      <c r="U1" s="78"/>
-      <c r="V1" s="78"/>
-      <c r="W1" s="78"/>
-      <c r="X1" s="78"/>
-      <c r="Y1" s="78"/>
-      <c r="Z1" s="78"/>
-      <c r="AA1" s="78"/>
-      <c r="AB1" s="78"/>
-      <c r="AC1" s="79"/>
-      <c r="AD1" s="79"/>
-      <c r="AE1" s="79"/>
-      <c r="AF1" s="79"/>
-      <c r="AG1" s="79"/>
-      <c r="AH1" s="79"/>
-      <c r="AI1" s="79"/>
-      <c r="AJ1" s="79"/>
-      <c r="AK1" s="79"/>
-      <c r="AL1" s="79"/>
-      <c r="AM1" s="79"/>
-      <c r="AN1" s="79"/>
-      <c r="AO1" s="79"/>
-      <c r="AP1" s="79"/>
-      <c r="AQ1" s="79"/>
-      <c r="AR1" s="79"/>
-      <c r="AS1" s="79"/>
-      <c r="AT1" s="79"/>
-      <c r="AU1" s="79"/>
-      <c r="AV1" s="79"/>
-      <c r="AW1" s="79"/>
-      <c r="AX1" s="79"/>
-      <c r="AY1" s="79"/>
-      <c r="AZ1" s="79"/>
-      <c r="BA1" s="79"/>
-      <c r="BB1" s="79"/>
-    </row>
-    <row r="2" spans="1:54" ht="16.5" customHeight="1">
+      <c r="B1" s="81"/>
+      <c r="C1" s="81"/>
+      <c r="D1" s="81"/>
+      <c r="E1" s="81"/>
+      <c r="F1" s="81"/>
+      <c r="G1" s="81"/>
+      <c r="H1" s="81"/>
+      <c r="I1" s="81"/>
+      <c r="J1" s="81"/>
+      <c r="K1" s="81"/>
+      <c r="L1" s="81"/>
+      <c r="M1" s="81"/>
+      <c r="N1" s="81"/>
+      <c r="O1" s="81"/>
+      <c r="P1" s="81"/>
+      <c r="Q1" s="81"/>
+      <c r="R1" s="81"/>
+      <c r="S1" s="81"/>
+      <c r="T1" s="81"/>
+      <c r="U1" s="81"/>
+      <c r="V1" s="81"/>
+      <c r="W1" s="81"/>
+      <c r="X1" s="81"/>
+      <c r="Y1" s="81"/>
+      <c r="Z1" s="81"/>
+      <c r="AA1" s="81"/>
+      <c r="AB1" s="81"/>
+      <c r="AC1" s="82"/>
+      <c r="AD1" s="82"/>
+      <c r="AE1" s="82"/>
+      <c r="AF1" s="82"/>
+      <c r="AG1" s="82"/>
+      <c r="AH1" s="82"/>
+      <c r="AI1" s="82"/>
+      <c r="AJ1" s="82"/>
+      <c r="AK1" s="82"/>
+      <c r="AL1" s="82"/>
+      <c r="AM1" s="82"/>
+      <c r="AN1" s="82"/>
+      <c r="AO1" s="82"/>
+      <c r="AP1" s="82"/>
+      <c r="AQ1" s="82"/>
+      <c r="AR1" s="82"/>
+      <c r="AS1" s="82"/>
+      <c r="AT1" s="82"/>
+      <c r="AU1" s="82"/>
+      <c r="AV1" s="82"/>
+      <c r="AW1" s="82"/>
+      <c r="AX1" s="82"/>
+      <c r="AY1" s="82"/>
+      <c r="AZ1" s="82"/>
+      <c r="BA1" s="82"/>
+      <c r="BB1" s="82"/>
+    </row>
+    <row r="2" spans="1:54" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="38"/>
       <c r="B2" s="39">
         <v>1980</v>
@@ -2435,7 +2446,7 @@
       <c r="BA2" s="45"/>
       <c r="BB2" s="46"/>
     </row>
-    <row r="3" spans="1:54" ht="16.5" customHeight="1">
+    <row r="3" spans="1:54" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="47" t="s">
         <v>65</v>
       </c>
@@ -2547,7 +2558,7 @@
       <c r="BA3" s="48"/>
       <c r="BB3" s="48"/>
     </row>
-    <row r="4" spans="1:54" ht="16.5" customHeight="1">
+    <row r="4" spans="1:54" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="50" t="s">
         <v>67</v>
       </c>
@@ -2659,7 +2670,7 @@
       <c r="BA4" s="52"/>
       <c r="BB4" s="52"/>
     </row>
-    <row r="5" spans="1:54" ht="16.5" customHeight="1">
+    <row r="5" spans="1:54" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="50" t="s">
         <v>68</v>
       </c>
@@ -2771,7 +2782,7 @@
       <c r="BA5" s="52"/>
       <c r="BB5" s="52"/>
     </row>
-    <row r="6" spans="1:54" ht="16.5" customHeight="1">
+    <row r="6" spans="1:54" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="50" t="s">
         <v>69</v>
       </c>
@@ -2883,7 +2894,7 @@
       <c r="BA6" s="52"/>
       <c r="BB6" s="52"/>
     </row>
-    <row r="7" spans="1:54" ht="16.5" customHeight="1">
+    <row r="7" spans="1:54" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="50" t="s">
         <v>70</v>
       </c>
@@ -2995,7 +3006,7 @@
       <c r="BA7" s="52"/>
       <c r="BB7" s="52"/>
     </row>
-    <row r="8" spans="1:54" ht="16.5" customHeight="1">
+    <row r="8" spans="1:54" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="50" t="s">
         <v>71</v>
       </c>
@@ -3107,7 +3118,7 @@
       <c r="BA8" s="52"/>
       <c r="BB8" s="52"/>
     </row>
-    <row r="9" spans="1:54" ht="16.5" customHeight="1">
+    <row r="9" spans="1:54" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="53" t="s">
         <v>72</v>
       </c>
@@ -3165,7 +3176,7 @@
       <c r="BA9" s="54"/>
       <c r="BB9" s="54"/>
     </row>
-    <row r="10" spans="1:54" ht="16.5" customHeight="1">
+    <row r="10" spans="1:54" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="50" t="s">
         <v>67</v>
       </c>
@@ -3279,7 +3290,7 @@
       <c r="BA10" s="56"/>
       <c r="BB10" s="56"/>
     </row>
-    <row r="11" spans="1:54" ht="16.5" customHeight="1">
+    <row r="11" spans="1:54" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="50" t="s">
         <v>68</v>
       </c>
@@ -3391,7 +3402,7 @@
       <c r="BA11" s="56"/>
       <c r="BB11" s="56"/>
     </row>
-    <row r="12" spans="1:54" ht="16.5" customHeight="1">
+    <row r="12" spans="1:54" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="50" t="s">
         <v>69</v>
       </c>
@@ -3503,7 +3514,7 @@
       <c r="BA12" s="56"/>
       <c r="BB12" s="56"/>
     </row>
-    <row r="13" spans="1:54" ht="16.5" customHeight="1">
+    <row r="13" spans="1:54" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="50" t="s">
         <v>70</v>
       </c>
@@ -3615,7 +3626,7 @@
       <c r="BA13" s="56"/>
       <c r="BB13" s="56"/>
     </row>
-    <row r="14" spans="1:54" ht="16.5" customHeight="1">
+    <row r="14" spans="1:54" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="50" t="s">
         <v>71</v>
       </c>
@@ -3727,7 +3738,7 @@
       <c r="BA14" s="56"/>
       <c r="BB14" s="56"/>
     </row>
-    <row r="15" spans="1:54" ht="16.5" customHeight="1">
+    <row r="15" spans="1:54" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="47" t="s">
         <v>73</v>
       </c>
@@ -3785,7 +3796,7 @@
       <c r="BA15" s="58"/>
       <c r="BB15" s="58"/>
     </row>
-    <row r="16" spans="1:54" ht="16.5" customHeight="1">
+    <row r="16" spans="1:54" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="50" t="s">
         <v>67</v>
       </c>
@@ -3897,7 +3908,7 @@
       <c r="BA16" s="59"/>
       <c r="BB16" s="59"/>
     </row>
-    <row r="17" spans="1:54" ht="16.5" customHeight="1">
+    <row r="17" spans="1:54" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="50" t="s">
         <v>68</v>
       </c>
@@ -4009,7 +4020,7 @@
       <c r="BA17" s="59"/>
       <c r="BB17" s="59"/>
     </row>
-    <row r="18" spans="1:54" ht="16.5" customHeight="1">
+    <row r="18" spans="1:54" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="50" t="s">
         <v>69</v>
       </c>
@@ -4121,7 +4132,7 @@
       <c r="BA18" s="59"/>
       <c r="BB18" s="59"/>
     </row>
-    <row r="19" spans="1:54" ht="16.5" customHeight="1">
+    <row r="19" spans="1:54" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="50" t="s">
         <v>70</v>
       </c>
@@ -4233,7 +4244,7 @@
       <c r="BA19" s="59"/>
       <c r="BB19" s="59"/>
     </row>
-    <row r="20" spans="1:54" ht="16.5" customHeight="1" thickBot="1">
+    <row r="20" spans="1:54" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A20" s="60" t="s">
         <v>71</v>
       </c>
@@ -4345,68 +4356,68 @@
       <c r="BA20" s="59"/>
       <c r="BB20" s="59"/>
     </row>
-    <row r="21" spans="1:54" s="63" customFormat="1" ht="12.75" customHeight="1">
-      <c r="A21" s="80" t="s">
+    <row r="21" spans="1:54" s="63" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="83" t="s">
         <v>74</v>
       </c>
-      <c r="B21" s="80"/>
-      <c r="C21" s="80"/>
-      <c r="D21" s="80"/>
-      <c r="E21" s="80"/>
-      <c r="F21" s="80"/>
-      <c r="G21" s="80"/>
-      <c r="H21" s="80"/>
-      <c r="I21" s="80"/>
-      <c r="J21" s="80"/>
-      <c r="K21" s="80"/>
-      <c r="L21" s="80"/>
-      <c r="M21" s="80"/>
-      <c r="N21" s="80"/>
-      <c r="O21" s="80"/>
-      <c r="P21" s="80"/>
-      <c r="Q21" s="80"/>
-    </row>
-    <row r="22" spans="1:54" s="63" customFormat="1" ht="12.75" customHeight="1">
-      <c r="A22" s="81"/>
-      <c r="B22" s="81"/>
-      <c r="C22" s="81"/>
-      <c r="D22" s="81"/>
-      <c r="E22" s="81"/>
-      <c r="F22" s="81"/>
-      <c r="G22" s="81"/>
-      <c r="H22" s="81"/>
-      <c r="I22" s="81"/>
-      <c r="J22" s="81"/>
-      <c r="K22" s="81"/>
-      <c r="L22" s="81"/>
-      <c r="M22" s="81"/>
-      <c r="N22" s="81"/>
-      <c r="O22" s="81"/>
-      <c r="P22" s="81"/>
-      <c r="Q22" s="81"/>
-    </row>
-    <row r="23" spans="1:54" s="63" customFormat="1" ht="12.75" customHeight="1">
-      <c r="A23" s="81" t="s">
+      <c r="B21" s="83"/>
+      <c r="C21" s="83"/>
+      <c r="D21" s="83"/>
+      <c r="E21" s="83"/>
+      <c r="F21" s="83"/>
+      <c r="G21" s="83"/>
+      <c r="H21" s="83"/>
+      <c r="I21" s="83"/>
+      <c r="J21" s="83"/>
+      <c r="K21" s="83"/>
+      <c r="L21" s="83"/>
+      <c r="M21" s="83"/>
+      <c r="N21" s="83"/>
+      <c r="O21" s="83"/>
+      <c r="P21" s="83"/>
+      <c r="Q21" s="83"/>
+    </row>
+    <row r="22" spans="1:54" s="63" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="84"/>
+      <c r="B22" s="84"/>
+      <c r="C22" s="84"/>
+      <c r="D22" s="84"/>
+      <c r="E22" s="84"/>
+      <c r="F22" s="84"/>
+      <c r="G22" s="84"/>
+      <c r="H22" s="84"/>
+      <c r="I22" s="84"/>
+      <c r="J22" s="84"/>
+      <c r="K22" s="84"/>
+      <c r="L22" s="84"/>
+      <c r="M22" s="84"/>
+      <c r="N22" s="84"/>
+      <c r="O22" s="84"/>
+      <c r="P22" s="84"/>
+      <c r="Q22" s="84"/>
+    </row>
+    <row r="23" spans="1:54" s="63" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="84" t="s">
         <v>75</v>
       </c>
-      <c r="B23" s="81"/>
-      <c r="C23" s="81"/>
-      <c r="D23" s="81"/>
-      <c r="E23" s="81"/>
-      <c r="F23" s="81"/>
-      <c r="G23" s="81"/>
-      <c r="H23" s="81"/>
-      <c r="I23" s="81"/>
-      <c r="J23" s="81"/>
-      <c r="K23" s="81"/>
-      <c r="L23" s="81"/>
-      <c r="M23" s="81"/>
-      <c r="N23" s="81"/>
-      <c r="O23" s="81"/>
-      <c r="P23" s="81"/>
-      <c r="Q23" s="81"/>
-    </row>
-    <row r="24" spans="1:54" s="63" customFormat="1" ht="12.75" customHeight="1">
+      <c r="B23" s="84"/>
+      <c r="C23" s="84"/>
+      <c r="D23" s="84"/>
+      <c r="E23" s="84"/>
+      <c r="F23" s="84"/>
+      <c r="G23" s="84"/>
+      <c r="H23" s="84"/>
+      <c r="I23" s="84"/>
+      <c r="J23" s="84"/>
+      <c r="K23" s="84"/>
+      <c r="L23" s="84"/>
+      <c r="M23" s="84"/>
+      <c r="N23" s="84"/>
+      <c r="O23" s="84"/>
+      <c r="P23" s="84"/>
+      <c r="Q23" s="84"/>
+    </row>
+    <row r="24" spans="1:54" s="63" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="77" t="s">
         <v>76</v>
       </c>
@@ -4427,7 +4438,7 @@
       <c r="P24" s="77"/>
       <c r="Q24" s="77"/>
     </row>
-    <row r="25" spans="1:54" s="63" customFormat="1" ht="12.75" customHeight="1">
+    <row r="25" spans="1:54" s="63" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="77" t="s">
         <v>77</v>
       </c>
@@ -4448,130 +4459,130 @@
       <c r="P25" s="77"/>
       <c r="Q25" s="77"/>
     </row>
-    <row r="26" spans="1:54" s="63" customFormat="1" ht="27.75" customHeight="1">
-      <c r="A26" s="82" t="s">
+    <row r="26" spans="1:54" s="63" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="78" t="s">
         <v>78</v>
       </c>
-      <c r="B26" s="82"/>
-      <c r="C26" s="82"/>
-      <c r="D26" s="82"/>
-      <c r="E26" s="82"/>
-      <c r="F26" s="82"/>
-      <c r="G26" s="82"/>
-      <c r="H26" s="82"/>
-      <c r="I26" s="82"/>
-      <c r="J26" s="82"/>
-      <c r="K26" s="82"/>
-      <c r="L26" s="82"/>
-      <c r="M26" s="82"/>
-      <c r="N26" s="82"/>
-      <c r="O26" s="82"/>
-      <c r="P26" s="82"/>
-      <c r="Q26" s="82"/>
-    </row>
-    <row r="27" spans="1:54" s="63" customFormat="1" ht="12.75" customHeight="1">
-      <c r="A27" s="82"/>
-      <c r="B27" s="82"/>
-      <c r="C27" s="82"/>
-      <c r="D27" s="82"/>
-      <c r="E27" s="82"/>
-      <c r="F27" s="82"/>
-      <c r="G27" s="82"/>
-      <c r="H27" s="82"/>
-      <c r="I27" s="82"/>
-      <c r="J27" s="82"/>
-      <c r="K27" s="82"/>
-      <c r="L27" s="82"/>
-      <c r="M27" s="82"/>
-      <c r="N27" s="82"/>
-      <c r="O27" s="82"/>
-      <c r="P27" s="82"/>
-      <c r="Q27" s="82"/>
-    </row>
-    <row r="28" spans="1:54" s="63" customFormat="1" ht="12.75" customHeight="1">
-      <c r="A28" s="83" t="s">
+      <c r="B26" s="78"/>
+      <c r="C26" s="78"/>
+      <c r="D26" s="78"/>
+      <c r="E26" s="78"/>
+      <c r="F26" s="78"/>
+      <c r="G26" s="78"/>
+      <c r="H26" s="78"/>
+      <c r="I26" s="78"/>
+      <c r="J26" s="78"/>
+      <c r="K26" s="78"/>
+      <c r="L26" s="78"/>
+      <c r="M26" s="78"/>
+      <c r="N26" s="78"/>
+      <c r="O26" s="78"/>
+      <c r="P26" s="78"/>
+      <c r="Q26" s="78"/>
+    </row>
+    <row r="27" spans="1:54" s="63" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="78"/>
+      <c r="B27" s="78"/>
+      <c r="C27" s="78"/>
+      <c r="D27" s="78"/>
+      <c r="E27" s="78"/>
+      <c r="F27" s="78"/>
+      <c r="G27" s="78"/>
+      <c r="H27" s="78"/>
+      <c r="I27" s="78"/>
+      <c r="J27" s="78"/>
+      <c r="K27" s="78"/>
+      <c r="L27" s="78"/>
+      <c r="M27" s="78"/>
+      <c r="N27" s="78"/>
+      <c r="O27" s="78"/>
+      <c r="P27" s="78"/>
+      <c r="Q27" s="78"/>
+    </row>
+    <row r="28" spans="1:54" s="63" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="79" t="s">
         <v>79</v>
       </c>
-      <c r="B28" s="83"/>
-      <c r="C28" s="83"/>
-      <c r="D28" s="83"/>
-      <c r="E28" s="83"/>
-      <c r="F28" s="83"/>
-      <c r="G28" s="83"/>
-      <c r="H28" s="83"/>
-      <c r="I28" s="83"/>
-      <c r="J28" s="83"/>
-      <c r="K28" s="83"/>
-      <c r="L28" s="83"/>
-      <c r="M28" s="83"/>
-      <c r="N28" s="83"/>
-      <c r="O28" s="83"/>
-      <c r="P28" s="83"/>
-      <c r="Q28" s="83"/>
-    </row>
-    <row r="29" spans="1:54" s="63" customFormat="1" ht="25.5" customHeight="1">
-      <c r="A29" s="84" t="s">
+      <c r="B28" s="79"/>
+      <c r="C28" s="79"/>
+      <c r="D28" s="79"/>
+      <c r="E28" s="79"/>
+      <c r="F28" s="79"/>
+      <c r="G28" s="79"/>
+      <c r="H28" s="79"/>
+      <c r="I28" s="79"/>
+      <c r="J28" s="79"/>
+      <c r="K28" s="79"/>
+      <c r="L28" s="79"/>
+      <c r="M28" s="79"/>
+      <c r="N28" s="79"/>
+      <c r="O28" s="79"/>
+      <c r="P28" s="79"/>
+      <c r="Q28" s="79"/>
+    </row>
+    <row r="29" spans="1:54" s="63" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="80" t="s">
         <v>80</v>
       </c>
-      <c r="B29" s="84"/>
-      <c r="C29" s="84"/>
-      <c r="D29" s="84"/>
-      <c r="E29" s="84"/>
-      <c r="F29" s="84"/>
-      <c r="G29" s="84"/>
-      <c r="H29" s="84"/>
-      <c r="I29" s="84"/>
-      <c r="J29" s="84"/>
-      <c r="K29" s="84"/>
-      <c r="L29" s="84"/>
-      <c r="M29" s="84"/>
-      <c r="N29" s="84"/>
-      <c r="O29" s="84"/>
-      <c r="P29" s="84"/>
-      <c r="Q29" s="84"/>
-    </row>
-    <row r="33" customFormat="1"/>
-    <row r="34" customFormat="1"/>
-    <row r="35" customFormat="1"/>
-    <row r="36" customFormat="1"/>
-    <row r="37" customFormat="1"/>
-    <row r="38" customFormat="1"/>
-    <row r="39" customFormat="1"/>
-    <row r="40" customFormat="1"/>
-    <row r="41" customFormat="1"/>
-    <row r="42" customFormat="1"/>
-    <row r="43" customFormat="1"/>
-    <row r="44" customFormat="1"/>
-    <row r="45" customFormat="1"/>
-    <row r="46" customFormat="1"/>
-    <row r="47" customFormat="1"/>
-    <row r="48" customFormat="1"/>
-    <row r="49" customFormat="1"/>
-    <row r="50" customFormat="1"/>
-    <row r="51" customFormat="1"/>
-    <row r="52" customFormat="1"/>
-    <row r="53" customFormat="1"/>
-    <row r="54" customFormat="1"/>
-    <row r="55" customFormat="1"/>
-    <row r="56" customFormat="1"/>
-    <row r="57" customFormat="1"/>
-    <row r="58" customFormat="1"/>
-    <row r="59" customFormat="1"/>
-    <row r="60" customFormat="1"/>
-    <row r="61" customFormat="1"/>
+      <c r="B29" s="80"/>
+      <c r="C29" s="80"/>
+      <c r="D29" s="80"/>
+      <c r="E29" s="80"/>
+      <c r="F29" s="80"/>
+      <c r="G29" s="80"/>
+      <c r="H29" s="80"/>
+      <c r="I29" s="80"/>
+      <c r="J29" s="80"/>
+      <c r="K29" s="80"/>
+      <c r="L29" s="80"/>
+      <c r="M29" s="80"/>
+      <c r="N29" s="80"/>
+      <c r="O29" s="80"/>
+      <c r="P29" s="80"/>
+      <c r="Q29" s="80"/>
+    </row>
+    <row r="33" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="34" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="35" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="36" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="37" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="38" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="39" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="40" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="41" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="42" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="43" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="44" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="45" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="46" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="47" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="48" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="49" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="50" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="51" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="52" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="53" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="54" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="55" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="56" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="57" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="58" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="59" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="60" customFormat="1" x14ac:dyDescent="0.3"/>
+    <row r="61" customFormat="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="A25:Q25"/>
-    <mergeCell ref="A26:Q26"/>
-    <mergeCell ref="A27:Q27"/>
-    <mergeCell ref="A28:Q28"/>
-    <mergeCell ref="A29:Q29"/>
     <mergeCell ref="A24:Q24"/>
     <mergeCell ref="A1:AB1"/>
     <mergeCell ref="AC1:BB1"/>
     <mergeCell ref="A21:Q21"/>
     <mergeCell ref="A22:Q22"/>
     <mergeCell ref="A23:Q23"/>
+    <mergeCell ref="A25:Q25"/>
+    <mergeCell ref="A26:Q26"/>
+    <mergeCell ref="A27:Q27"/>
+    <mergeCell ref="A28:Q28"/>
+    <mergeCell ref="A29:Q29"/>
   </mergeCells>
   <phoneticPr fontId="38" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4581,17 +4592,17 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:E48"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="9.125" defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="30.109375" style="3" customWidth="1"/>
-    <col min="2" max="2" width="29.88671875" style="3" customWidth="1"/>
-    <col min="3" max="3" width="25.21875" style="3" customWidth="1"/>
-    <col min="4" max="4" width="22.77734375" style="3" customWidth="1"/>
-    <col min="5" max="5" width="25.109375" style="3" customWidth="1"/>
-    <col min="6" max="16384" width="9.109375" style="3"/>
+    <col min="1" max="1" width="30.125" style="3" customWidth="1"/>
+    <col min="2" max="2" width="29.875" style="3" customWidth="1"/>
+    <col min="3" max="3" width="25.25" style="3" customWidth="1"/>
+    <col min="4" max="4" width="22.75" style="3" customWidth="1"/>
+    <col min="5" max="5" width="25.125" style="3" customWidth="1"/>
+    <col min="6" max="16384" width="9.125" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" customFormat="1" ht="15" thickBot="1">
+    <row r="1" spans="1:5" customFormat="1" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
         <v>52</v>
       </c>
@@ -4600,7 +4611,7 @@
       <c r="D1" s="33"/>
       <c r="E1" s="33"/>
     </row>
-    <row r="2" spans="1:5" s="2" customFormat="1" ht="57.6">
+    <row r="2" spans="1:5" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -4617,7 +4628,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="15" thickBot="1">
+    <row r="3" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="3">
         <v>13</v>
       </c>
@@ -4637,12 +4648,12 @@
         <v>13.378781688359696</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="15" thickBot="1">
+    <row r="5" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="10" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="28.8">
+    <row r="6" spans="1:5" ht="33" x14ac:dyDescent="0.3">
       <c r="A6" s="7" t="s">
         <v>59</v>
       </c>
@@ -4657,7 +4668,7 @@
       </c>
       <c r="E6" s="2"/>
     </row>
-    <row r="7" spans="1:5" ht="15" thickBot="1">
+    <row r="7" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="68">
         <v>28</v>
       </c>
@@ -4672,7 +4683,7 @@
       </c>
       <c r="E7" s="67"/>
     </row>
-    <row r="10" spans="1:5">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" s="10" t="s">
         <v>56</v>
       </c>
@@ -4681,14 +4692,14 @@
       <c r="D10" s="34"/>
       <c r="E10" s="34"/>
     </row>
-    <row r="11" spans="1:5" s="9" customFormat="1">
+    <row r="11" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A11" s="15" t="s">
         <v>33</v>
       </c>
       <c r="B11" s="14"/>
       <c r="C11" s="15"/>
     </row>
-    <row r="12" spans="1:5" s="9" customFormat="1">
+    <row r="12" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A12" s="9" t="s">
         <v>34</v>
       </c>
@@ -4696,7 +4707,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="13" spans="1:5" s="9" customFormat="1">
+    <row r="13" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A13" s="9" t="s">
         <v>36</v>
       </c>
@@ -4704,7 +4715,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="14" spans="1:5" s="9" customFormat="1" ht="15" thickBot="1">
+    <row r="14" spans="1:5" s="9" customFormat="1" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="9" t="s">
         <v>38</v>
       </c>
@@ -4712,17 +4723,17 @@
         <v>39</v>
       </c>
     </row>
-    <row r="15" spans="1:5" s="9" customFormat="1">
+    <row r="15" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A15" s="17" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="16" spans="1:5" s="9" customFormat="1" ht="15" thickBot="1">
+    <row r="16" spans="1:5" s="9" customFormat="1" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="18">
         <v>24</v>
       </c>
     </row>
-    <row r="18" spans="1:5">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" s="10" t="s">
         <v>21</v>
       </c>
@@ -4731,7 +4742,7 @@
       <c r="D18" s="34"/>
       <c r="E18" s="34"/>
     </row>
-    <row r="19" spans="1:5">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" s="15" t="s">
         <v>10</v>
       </c>
@@ -4742,7 +4753,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="20" spans="1:5">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>22</v>
       </c>
@@ -4753,7 +4764,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="21" spans="1:5" ht="15" thickBot="1">
+    <row r="21" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>24</v>
       </c>
@@ -4764,7 +4775,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="22" spans="1:5" ht="15" thickBot="1">
+    <row r="22" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A22"/>
       <c r="B22" s="11" t="s">
         <v>26</v>
@@ -4773,17 +4784,17 @@
         <v>34</v>
       </c>
     </row>
-    <row r="23" spans="1:5">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="24" spans="1:5">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="26" spans="1:5">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" s="10" t="s">
         <v>13</v>
       </c>
@@ -4792,7 +4803,7 @@
       <c r="D26" s="34"/>
       <c r="E26" s="34"/>
     </row>
-    <row r="27" spans="1:5" ht="15" thickBot="1">
+    <row r="27" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A27" s="15" t="s">
         <v>10</v>
       </c>
@@ -4803,7 +4814,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="28" spans="1:5" ht="15" thickBot="1">
+    <row r="28" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>14</v>
       </c>
@@ -4814,7 +4825,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="30" spans="1:5" ht="15" thickBot="1">
+    <row r="30" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A30" s="10" t="s">
         <v>58</v>
       </c>
@@ -4823,7 +4834,7 @@
       <c r="D30" s="34"/>
       <c r="E30" s="34"/>
     </row>
-    <row r="31" spans="1:5" ht="28.8">
+    <row r="31" spans="1:5" ht="33" x14ac:dyDescent="0.3">
       <c r="A31" s="21" t="s">
         <v>43</v>
       </c>
@@ -4840,7 +4851,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="32" spans="1:5">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32" s="20">
         <v>1997</v>
       </c>
@@ -4853,7 +4864,7 @@
       <c r="D32" s="9"/>
       <c r="E32" s="9"/>
     </row>
-    <row r="33" spans="1:5">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" s="20">
         <v>1998</v>
       </c>
@@ -4872,7 +4883,7 @@
         <v>6.6484424338501588E-2</v>
       </c>
     </row>
-    <row r="34" spans="1:5">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" s="20">
         <v>1999</v>
       </c>
@@ -4891,7 +4902,7 @@
         <v>2.9143636995467476E-2</v>
       </c>
     </row>
-    <row r="35" spans="1:5">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35" s="20">
         <v>2000</v>
       </c>
@@ -4910,7 +4921,7 @@
         <v>6.8191523924614153E-2</v>
       </c>
     </row>
-    <row r="36" spans="1:5">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36" s="20">
         <v>2001</v>
       </c>
@@ -4929,7 +4940,7 @@
         <v>4.0815360868813244E-3</v>
       </c>
     </row>
-    <row r="37" spans="1:5">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A37" s="20">
         <v>2002</v>
       </c>
@@ -4948,7 +4959,7 @@
         <v>0.10769048766665149</v>
       </c>
     </row>
-    <row r="38" spans="1:5">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A38" s="20">
         <v>2003</v>
       </c>
@@ -4967,7 +4978,7 @@
         <v>5.9053805049687755E-2</v>
       </c>
     </row>
-    <row r="39" spans="1:5">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A39" s="20">
         <v>2004</v>
       </c>
@@ -4986,7 +4997,7 @@
         <v>5.8670234757052138E-2</v>
       </c>
     </row>
-    <row r="40" spans="1:5">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A40" s="20">
         <v>2005</v>
       </c>
@@ -5005,7 +5016,7 @@
         <v>6.1781753631599455E-2</v>
       </c>
     </row>
-    <row r="41" spans="1:5">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A41" s="20">
         <v>2006</v>
       </c>
@@ -5024,7 +5035,7 @@
         <v>6.5906687839630079E-2</v>
       </c>
     </row>
-    <row r="42" spans="1:5" ht="15" thickBot="1">
+    <row r="42" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A42" s="25">
         <v>2007</v>
       </c>
@@ -5043,14 +5054,14 @@
         <v>5.9604038733197397E-2</v>
       </c>
     </row>
-    <row r="43" spans="1:5">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A43"/>
       <c r="B43"/>
       <c r="C43"/>
       <c r="D43"/>
       <c r="E43"/>
     </row>
-    <row r="44" spans="1:5">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A44" s="1" t="s">
         <v>47</v>
       </c>
@@ -5058,7 +5069,7 @@
       <c r="C44"/>
       <c r="D44"/>
     </row>
-    <row r="45" spans="1:5">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A45" s="28">
         <f>AVERAGE(E33:E42)</f>
         <v>5.8060812902328285E-2</v>
@@ -5067,13 +5078,13 @@
       <c r="C45"/>
       <c r="D45"/>
     </row>
-    <row r="46" spans="1:5" ht="15" thickBot="1">
+    <row r="46" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A46"/>
       <c r="B46"/>
       <c r="C46"/>
       <c r="D46"/>
     </row>
-    <row r="47" spans="1:5" ht="28.8">
+    <row r="47" spans="1:5" ht="33" x14ac:dyDescent="0.3">
       <c r="A47" s="36" t="s">
         <v>48</v>
       </c>
@@ -5081,7 +5092,7 @@
       <c r="C47"/>
       <c r="D47"/>
     </row>
-    <row r="48" spans="1:5" ht="15" thickBot="1">
+    <row r="48" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A48" s="35">
         <f>1/A45</f>
         <v>17.22332068760786</v>
@@ -5101,25 +5112,25 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD149825-14BA-415D-91AD-354F00EEF420}">
-  <dimension ref="A1:J40"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
+  <dimension ref="A1:K40"/>
+  <sheetFormatPr defaultColWidth="8.75" defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="19.109375" style="70" customWidth="1"/>
-    <col min="2" max="2" width="11.109375" style="70" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="10.109375" style="70" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="12.44140625" style="70" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.109375" style="70" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.44140625" style="70" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.109375" style="70" bestFit="1" customWidth="1"/>
-    <col min="10" max="16384" width="8.77734375" style="70"/>
+    <col min="1" max="1" width="19.125" style="70" customWidth="1"/>
+    <col min="2" max="2" width="11.125" style="70" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="10.125" style="70" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="12.5" style="70" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.125" style="70" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.5" style="70" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.125" style="70" bestFit="1" customWidth="1"/>
+    <col min="10" max="16384" width="8.75" style="70"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="70" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B2" s="70" t="s">
         <v>101</v>
       </c>
@@ -5145,7 +5156,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="3" spans="1:9">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B3" s="70" t="s">
         <v>52</v>
       </c>
@@ -5171,7 +5182,7 @@
         <v>7728.5710293009906</v>
       </c>
     </row>
-    <row r="4" spans="1:9">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B4" s="70" t="s">
         <v>55</v>
       </c>
@@ -5197,7 +5208,7 @@
         <v>3161.4504274369956</v>
       </c>
     </row>
-    <row r="5" spans="1:9">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B5" s="70" t="s">
         <v>56</v>
       </c>
@@ -5223,7 +5234,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:9">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B6" s="70" t="s">
         <v>21</v>
       </c>
@@ -5249,7 +5260,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:9">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B7" s="70" t="s">
         <v>13</v>
       </c>
@@ -5275,7 +5286,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:9">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B8" s="70" t="s">
         <v>58</v>
       </c>
@@ -5301,12 +5312,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:9">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" s="70" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="11" spans="1:9">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B11" s="70" t="s">
         <v>101</v>
       </c>
@@ -5332,7 +5343,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="12" spans="1:9">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B12" s="70" t="s">
         <v>52</v>
       </c>
@@ -5358,7 +5369,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:9">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B13" s="70" t="s">
         <v>55</v>
       </c>
@@ -5384,7 +5395,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:9">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B14" s="70" t="s">
         <v>56</v>
       </c>
@@ -5410,7 +5421,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:9">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B15" s="70" t="s">
         <v>21</v>
       </c>
@@ -5436,7 +5447,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:9">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B16" s="70" t="s">
         <v>13</v>
       </c>
@@ -5462,7 +5473,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:9">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B17" s="70" t="s">
         <v>58</v>
       </c>
@@ -5488,12 +5499,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:9">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20" s="70" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="22" spans="1:9">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B22" s="70">
         <v>2019</v>
       </c>
@@ -5501,7 +5512,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="23" spans="1:9">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A23" s="70" t="s">
         <v>111</v>
       </c>
@@ -5517,7 +5528,7 @@
         <v>11.724644713881862</v>
       </c>
     </row>
-    <row r="24" spans="1:9">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A24" s="70" t="s">
         <v>112</v>
       </c>
@@ -5533,7 +5544,7 @@
         <v>11.325209578137313</v>
       </c>
     </row>
-    <row r="25" spans="1:9">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A25" s="70" t="s">
         <v>113</v>
       </c>
@@ -5545,7 +5556,7 @@
         <v>0.27844474080318277</v>
       </c>
     </row>
-    <row r="26" spans="1:9">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A26" s="70" t="s">
         <v>114</v>
       </c>
@@ -5557,13 +5568,13 @@
         <v>0.38904941180819808</v>
       </c>
     </row>
-    <row r="27" spans="1:9">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C27" s="72"/>
     </row>
-    <row r="28" spans="1:9">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C28" s="72"/>
     </row>
-    <row r="29" spans="1:9">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A29" s="70" t="s">
         <v>115</v>
       </c>
@@ -5579,7 +5590,7 @@
         <v>20.43541033331925</v>
       </c>
     </row>
-    <row r="30" spans="1:9">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A30" s="70" t="s">
         <v>116</v>
       </c>
@@ -5595,7 +5606,7 @@
         <v>13.907940419258974</v>
       </c>
     </row>
-    <row r="31" spans="1:9">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A31" s="70" t="s">
         <v>117</v>
       </c>
@@ -5607,7 +5618,7 @@
         <v>6.8718275287445466E-2</v>
       </c>
     </row>
-    <row r="32" spans="1:9">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A32" s="70" t="s">
         <v>118</v>
       </c>
@@ -5619,7 +5630,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="34" spans="1:10">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A34" s="74" t="s">
         <v>128</v>
       </c>
@@ -5630,7 +5641,7 @@
       <c r="F34" s="74"/>
       <c r="G34" s="74"/>
     </row>
-    <row r="35" spans="1:10">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A35" s="74"/>
       <c r="B35" s="74">
         <v>2000</v>
@@ -5650,8 +5661,10 @@
       <c r="G35" s="74">
         <v>2021</v>
       </c>
-    </row>
-    <row r="36" spans="1:10">
+      <c r="J35" s="3"/>
+      <c r="K35" s="3"/>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A36" s="74" t="s">
         <v>121</v>
       </c>
@@ -5673,15 +5686,15 @@
       <c r="G36" s="76">
         <v>15.6</v>
       </c>
+      <c r="H36" s="70" t="s">
+        <v>126</v>
+      </c>
       <c r="I36" s="74" t="s">
-        <v>126</v>
-      </c>
-      <c r="J36" s="75">
-        <f>AVERAGE(F36:F37)</f>
-        <v>15.4</v>
-      </c>
-    </row>
-    <row r="37" spans="1:10">
+        <v>129</v>
+      </c>
+      <c r="J36" s="75"/>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A37" s="74" t="s">
         <v>122</v>
       </c>
@@ -5703,15 +5716,15 @@
       <c r="G37" s="76">
         <v>15.5</v>
       </c>
+      <c r="H37" s="70" t="s">
+        <v>127</v>
+      </c>
       <c r="I37" s="75" t="s">
-        <v>127</v>
-      </c>
-      <c r="J37" s="75">
-        <f>AVERAGE(F38:F39)</f>
-        <v>16.8</v>
-      </c>
-    </row>
-    <row r="38" spans="1:10">
+        <v>129</v>
+      </c>
+      <c r="J37" s="75"/>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A38" s="74" t="s">
         <v>123</v>
       </c>
@@ -5733,8 +5746,14 @@
       <c r="G38" s="76">
         <v>17.3</v>
       </c>
-    </row>
-    <row r="39" spans="1:10">
+      <c r="H38" s="70" t="s">
+        <v>130</v>
+      </c>
+      <c r="I38" s="70" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A39" s="74" t="s">
         <v>124</v>
       </c>
@@ -5756,8 +5775,14 @@
       <c r="G39" s="76">
         <v>18.2</v>
       </c>
-    </row>
-    <row r="40" spans="1:10">
+      <c r="H39" s="70" t="s">
+        <v>130</v>
+      </c>
+      <c r="I39" s="70" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A40" s="74" t="s">
         <v>125</v>
       </c>
@@ -5793,14 +5818,14 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.6640625" customWidth="1"/>
+    <col min="1" max="1" width="14.625" customWidth="1"/>
     <col min="2" max="2" width="19" customWidth="1"/>
-    <col min="3" max="3" width="15.6640625" customWidth="1"/>
+    <col min="3" max="3" width="15.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="28.8">
+    <row r="1" spans="1:3" ht="33" x14ac:dyDescent="0.3">
       <c r="A1" s="69" t="s">
         <v>100</v>
       </c>
@@ -5811,33 +5836,33 @@
         <v>93</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>52</v>
       </c>
       <c r="B2" s="73">
-        <f>'SK calcs'!J36</f>
-        <v>15.4</v>
+        <f>'SK calcs'!G36</f>
+        <v>15.6</v>
       </c>
       <c r="C2" s="73">
-        <f t="shared" ref="C2:C7" si="0">B2</f>
-        <v>15.4</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
+        <f>AVERAGE('SK calcs'!$G$38:$G$39)</f>
+        <v>17.75</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>55</v>
       </c>
       <c r="B3" s="73">
-        <f>'SK calcs'!J37</f>
-        <v>16.8</v>
+        <f>'SK calcs'!G37</f>
+        <v>15.5</v>
       </c>
       <c r="C3" s="73">
-        <f t="shared" si="0"/>
-        <v>16.8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3">
+        <f>AVERAGE('SK calcs'!$G$38:$G$39)</f>
+        <v>17.75</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>56</v>
       </c>
@@ -5846,11 +5871,11 @@
         <v>24</v>
       </c>
       <c r="C4" s="37">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="C2:C7" si="0">B4</f>
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="1:3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>21</v>
       </c>
@@ -5863,7 +5888,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="6" spans="1:3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>13</v>
       </c>
@@ -5876,7 +5901,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="7" spans="1:3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>58</v>
       </c>
@@ -5896,15 +5921,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100E59C87379D9A4242BB3A95F198D6F941" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="07a235b40ffe2d9a960bde50f6511605">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="40f4d404-d193-41dc-bb72-733c1e774208" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="485fc8e6f691b86ce0aee9b7e82feca0" ns2:_="">
     <xsd:import namespace="40f4d404-d193-41dc-bb72-733c1e774208"/>
@@ -6048,6 +6064,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement/>
@@ -6055,14 +6080,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{48C589ED-403D-43C7-8D67-619C9CBC31EC}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{26A9F799-6530-441C-9A49-116D487C0166}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -6076,6 +6093,14 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{48C589ED-403D-43C7-8D67-619C9CBC31EC}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Transport calibration push, pending review from NextGroup
</commit_message>
<xml_diff>
--- a/InputData/trans/AVL/Avg Vehicle Lifetime.xlsx
+++ b/InputData/trans/AVL/Avg Vehicle Lifetime.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\administer\Dropbox\kjh\2026\01.EPS\01.EI\01.메일\260108_메일회신\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanOBrien\Models\EPS\SK\eps-southkorea\InputData\trans\AVL\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1944F64F-AD81-4996-A4B5-75E70CAE79BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C569AA2F-C350-4EDA-85E0-CDF30FF8D608}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-25260" yWindow="1515" windowWidth="24345" windowHeight="13980" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="9" r:id="rId1"/>
@@ -19,7 +19,7 @@
     <sheet name="SK calcs" sheetId="12" r:id="rId4"/>
     <sheet name="AVL" sheetId="10" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="191029" iterate="1" iterateDelta="1.0000000000000001E-5"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="133">
   <si>
     <t>Car Avg Lifetime, years (Page 22, Table 7)</t>
   </si>
@@ -475,27 +475,30 @@
     <t>freight</t>
     <phoneticPr fontId="38" type="noConversion"/>
   </si>
+  <si>
+    <t>Passenger LDVs lifetime calculated by calibration</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
   <numFmts count="9">
-    <numFmt numFmtId="176" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="177" formatCode="###0.00_)"/>
-    <numFmt numFmtId="178" formatCode="\(\R\)General"/>
-    <numFmt numFmtId="179" formatCode="\(\R\)\ ###0"/>
-    <numFmt numFmtId="180" formatCode="0.0"/>
-    <numFmt numFmtId="181" formatCode="\(\R\)0.0"/>
-    <numFmt numFmtId="182" formatCode="#,##0_)"/>
-    <numFmt numFmtId="183" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="184" formatCode="_(* #,##0.0_);_(* \(#,##0.0\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="###0.00_)"/>
+    <numFmt numFmtId="165" formatCode="\(\R\)General"/>
+    <numFmt numFmtId="166" formatCode="\(\R\)\ ###0"/>
+    <numFmt numFmtId="167" formatCode="0.0"/>
+    <numFmt numFmtId="168" formatCode="\(\R\)0.0"/>
+    <numFmt numFmtId="169" formatCode="#,##0_)"/>
+    <numFmt numFmtId="170" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="171" formatCode="_(* #,##0.0_);_(* \(#,##0.0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="40" x14ac:knownFonts="1">
+  <fonts count="40">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -503,7 +506,7 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -511,7 +514,7 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -519,14 +522,14 @@
       <b/>
       <sz val="9"/>
       <color theme="1"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="9"/>
       <color theme="1"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -534,7 +537,7 @@
       <u/>
       <sz val="10"/>
       <color theme="4"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -549,7 +552,7 @@
       <b/>
       <sz val="12"/>
       <color theme="4"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -566,14 +569,14 @@
       <i/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -581,7 +584,7 @@
       <b/>
       <sz val="18"/>
       <color theme="3"/>
-      <name val="맑은 고딕"/>
+      <name val="Cambria"/>
       <family val="2"/>
       <scheme val="major"/>
     </font>
@@ -589,7 +592,7 @@
       <b/>
       <sz val="15"/>
       <color theme="3"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -597,7 +600,7 @@
       <b/>
       <sz val="13"/>
       <color theme="3"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -605,35 +608,35 @@
       <b/>
       <sz val="11"/>
       <color theme="3"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF006100"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF9C0006"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF9C6500"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF3F3F76"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -641,7 +644,7 @@
       <b/>
       <sz val="11"/>
       <color rgb="FF3F3F3F"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -649,14 +652,14 @@
       <b/>
       <sz val="11"/>
       <color rgb="FFFA7D00"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FFFA7D00"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -664,14 +667,14 @@
       <b/>
       <sz val="11"/>
       <color theme="0"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -679,21 +682,21 @@
       <i/>
       <sz val="11"/>
       <color rgb="FF7F7F7F"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="0"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -750,13 +753,13 @@
       <i/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="8"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="129"/>
       <scheme val="minor"/>
@@ -764,7 +767,7 @@
     <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="129"/>
       <scheme val="minor"/>
@@ -1342,7 +1345,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyProtection="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="177" fontId="8" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="10">
@@ -1399,10 +1402,10 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="10">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="182" fontId="33" fillId="0" borderId="10">
+    <xf numFmtId="169" fontId="33" fillId="0" borderId="10">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="85">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -1507,10 +1510,10 @@
     <xf numFmtId="1" fontId="30" fillId="0" borderId="29" xfId="59" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="178" fontId="30" fillId="0" borderId="29" xfId="59" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="30" fillId="0" borderId="29" xfId="59" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="178" fontId="30" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="30" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="29" xfId="59" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1522,7 +1525,7 @@
     <xf numFmtId="1" fontId="30" fillId="0" borderId="0" xfId="59" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="179" fontId="30" fillId="0" borderId="0" xfId="59" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="30" fillId="0" borderId="0" xfId="59" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1542,21 +1545,21 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="3" fontId="31" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="180" fontId="30" fillId="0" borderId="0" xfId="60" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="30" fillId="0" borderId="0" xfId="60" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="180" fontId="31" fillId="0" borderId="0" xfId="16" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="180" fontId="31" fillId="0" borderId="0" xfId="16" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="181" fontId="31" fillId="0" borderId="0" xfId="16" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="167" fontId="31" fillId="0" borderId="0" xfId="16" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="167" fontId="31" fillId="0" borderId="0" xfId="16" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="168" fontId="31" fillId="0" borderId="0" xfId="16" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="3" fontId="31" fillId="0" borderId="0" xfId="61" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="180" fontId="31" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="167" fontId="31" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="31" fillId="0" borderId="27" xfId="60" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
     </xf>
-    <xf numFmtId="180" fontId="31" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="31" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="31" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1579,16 +1582,28 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="183" fontId="0" fillId="0" borderId="0" xfId="62" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="183" fontId="37" fillId="0" borderId="0" xfId="62" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="62" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="170" fontId="37" fillId="0" borderId="0" xfId="62" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="9" fontId="0" fillId="36" borderId="0" xfId="16" applyFont="1" applyFill="1"/>
     <xf numFmtId="1" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="183" fontId="24" fillId="0" borderId="0" xfId="62" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="183" fontId="39" fillId="0" borderId="0" xfId="62" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="184" fontId="39" fillId="0" borderId="0" xfId="62" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="170" fontId="24" fillId="0" borderId="0" xfId="62" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="170" fontId="39" fillId="0" borderId="0" xfId="62" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="171" fontId="39" fillId="0" borderId="0" xfId="62" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="35" fillId="0" borderId="0" xfId="15" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="27" xfId="58" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="58" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="22" xfId="15" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="15" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1598,83 +1613,71 @@
     <xf numFmtId="0" fontId="35" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="27" xfId="58" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="58" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="22" xfId="15" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="15" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="63">
-    <cellStyle name="20% - 강조색1" xfId="35" builtinId="30" customBuiltin="1"/>
-    <cellStyle name="20% - 강조색2" xfId="39" builtinId="34" customBuiltin="1"/>
-    <cellStyle name="20% - 강조색3" xfId="43" builtinId="38" customBuiltin="1"/>
-    <cellStyle name="20% - 강조색4" xfId="47" builtinId="42" customBuiltin="1"/>
-    <cellStyle name="20% - 강조색5" xfId="51" builtinId="46" customBuiltin="1"/>
-    <cellStyle name="20% - 강조색6" xfId="55" builtinId="50" customBuiltin="1"/>
-    <cellStyle name="40% - 강조색1" xfId="36" builtinId="31" customBuiltin="1"/>
-    <cellStyle name="40% - 강조색2" xfId="40" builtinId="35" customBuiltin="1"/>
-    <cellStyle name="40% - 강조색3" xfId="44" builtinId="39" customBuiltin="1"/>
-    <cellStyle name="40% - 강조색4" xfId="48" builtinId="43" customBuiltin="1"/>
-    <cellStyle name="40% - 강조색5" xfId="52" builtinId="47" customBuiltin="1"/>
-    <cellStyle name="40% - 강조색6" xfId="56" builtinId="51" customBuiltin="1"/>
-    <cellStyle name="60% - 강조색1" xfId="37" builtinId="32" customBuiltin="1"/>
-    <cellStyle name="60% - 강조색2" xfId="41" builtinId="36" customBuiltin="1"/>
-    <cellStyle name="60% - 강조색3" xfId="45" builtinId="40" customBuiltin="1"/>
-    <cellStyle name="60% - 강조색4" xfId="49" builtinId="44" customBuiltin="1"/>
-    <cellStyle name="60% - 강조색5" xfId="53" builtinId="48" customBuiltin="1"/>
-    <cellStyle name="60% - 강조색6" xfId="57" builtinId="52" customBuiltin="1"/>
+    <cellStyle name="20% - Accent1" xfId="35" builtinId="30" customBuiltin="1"/>
+    <cellStyle name="20% - Accent2" xfId="39" builtinId="34" customBuiltin="1"/>
+    <cellStyle name="20% - Accent3" xfId="43" builtinId="38" customBuiltin="1"/>
+    <cellStyle name="20% - Accent4" xfId="47" builtinId="42" customBuiltin="1"/>
+    <cellStyle name="20% - Accent5" xfId="51" builtinId="46" customBuiltin="1"/>
+    <cellStyle name="20% - Accent6" xfId="55" builtinId="50" customBuiltin="1"/>
+    <cellStyle name="40% - Accent1" xfId="36" builtinId="31" customBuiltin="1"/>
+    <cellStyle name="40% - Accent2" xfId="40" builtinId="35" customBuiltin="1"/>
+    <cellStyle name="40% - Accent3" xfId="44" builtinId="39" customBuiltin="1"/>
+    <cellStyle name="40% - Accent4" xfId="48" builtinId="43" customBuiltin="1"/>
+    <cellStyle name="40% - Accent5" xfId="52" builtinId="47" customBuiltin="1"/>
+    <cellStyle name="40% - Accent6" xfId="56" builtinId="51" customBuiltin="1"/>
+    <cellStyle name="60% - Accent1" xfId="37" builtinId="32" customBuiltin="1"/>
+    <cellStyle name="60% - Accent2" xfId="41" builtinId="36" customBuiltin="1"/>
+    <cellStyle name="60% - Accent3" xfId="45" builtinId="40" customBuiltin="1"/>
+    <cellStyle name="60% - Accent4" xfId="49" builtinId="44" customBuiltin="1"/>
+    <cellStyle name="60% - Accent5" xfId="53" builtinId="48" customBuiltin="1"/>
+    <cellStyle name="60% - Accent6" xfId="57" builtinId="52" customBuiltin="1"/>
+    <cellStyle name="Accent1" xfId="34" builtinId="29" customBuiltin="1"/>
+    <cellStyle name="Accent2" xfId="38" builtinId="33" customBuiltin="1"/>
+    <cellStyle name="Accent3" xfId="42" builtinId="37" customBuiltin="1"/>
+    <cellStyle name="Accent4" xfId="46" builtinId="41" customBuiltin="1"/>
+    <cellStyle name="Accent5" xfId="50" builtinId="45" customBuiltin="1"/>
+    <cellStyle name="Accent6" xfId="54" builtinId="49" customBuiltin="1"/>
+    <cellStyle name="Bad" xfId="23" builtinId="27" customBuiltin="1"/>
     <cellStyle name="Body: normal cell" xfId="3" xr:uid="{00000000-0005-0000-0000-000019000000}"/>
+    <cellStyle name="Calculation" xfId="27" builtinId="22" customBuiltin="1"/>
+    <cellStyle name="Check Cell" xfId="29" builtinId="23" customBuiltin="1"/>
+    <cellStyle name="Comma" xfId="62" builtinId="3"/>
     <cellStyle name="Data" xfId="14" xr:uid="{00000000-0005-0000-0000-00001C000000}"/>
     <cellStyle name="Data no deci" xfId="61" xr:uid="{00000000-0005-0000-0000-00001D000000}"/>
+    <cellStyle name="Explanatory Text" xfId="32" builtinId="53" customBuiltin="1"/>
+    <cellStyle name="Followed Hyperlink" xfId="11" builtinId="9" customBuiltin="1"/>
     <cellStyle name="Font: Calibri, 9pt regular" xfId="9" xr:uid="{00000000-0005-0000-0000-000020000000}"/>
     <cellStyle name="Footnotes: all except top row" xfId="12" xr:uid="{00000000-0005-0000-0000-000021000000}"/>
     <cellStyle name="Footnotes: top row" xfId="7" xr:uid="{00000000-0005-0000-0000-000022000000}"/>
+    <cellStyle name="Good" xfId="22" builtinId="26" customBuiltin="1"/>
     <cellStyle name="Header: bottom row" xfId="2" xr:uid="{00000000-0005-0000-0000-000024000000}"/>
     <cellStyle name="Header: top rows" xfId="4" xr:uid="{00000000-0005-0000-0000-000025000000}"/>
+    <cellStyle name="Heading 1" xfId="18" builtinId="16" customBuiltin="1"/>
+    <cellStyle name="Heading 2" xfId="19" builtinId="17" customBuiltin="1"/>
+    <cellStyle name="Heading 3" xfId="20" builtinId="18" customBuiltin="1"/>
+    <cellStyle name="Heading 4" xfId="21" builtinId="19" customBuiltin="1"/>
     <cellStyle name="Hed Side" xfId="15" xr:uid="{00000000-0005-0000-0000-00002A000000}"/>
     <cellStyle name="Hed Side Regular" xfId="60" xr:uid="{00000000-0005-0000-0000-00002B000000}"/>
     <cellStyle name="Hed Top" xfId="59" xr:uid="{00000000-0005-0000-0000-00002C000000}"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Hyperlink 2" xfId="10" xr:uid="{00000000-0005-0000-0000-00002E000000}"/>
+    <cellStyle name="Input" xfId="25" builtinId="20" customBuiltin="1"/>
+    <cellStyle name="Linked Cell" xfId="28" builtinId="24" customBuiltin="1"/>
+    <cellStyle name="Neutral" xfId="24" builtinId="28" customBuiltin="1"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Note" xfId="31" builtinId="10" customBuiltin="1"/>
+    <cellStyle name="Output" xfId="26" builtinId="21" customBuiltin="1"/>
     <cellStyle name="Parent row" xfId="6" xr:uid="{00000000-0005-0000-0000-000035000000}"/>
+    <cellStyle name="Percent" xfId="16" builtinId="5"/>
     <cellStyle name="Section Break" xfId="8" xr:uid="{00000000-0005-0000-0000-000037000000}"/>
     <cellStyle name="Section Break: parent row" xfId="5" xr:uid="{00000000-0005-0000-0000-000038000000}"/>
     <cellStyle name="Table title" xfId="13" xr:uid="{00000000-0005-0000-0000-000039000000}"/>
+    <cellStyle name="Title" xfId="17" builtinId="15" customBuiltin="1"/>
     <cellStyle name="Title-2" xfId="58" xr:uid="{00000000-0005-0000-0000-00003B000000}"/>
-    <cellStyle name="강조색1" xfId="34" builtinId="29" customBuiltin="1"/>
-    <cellStyle name="강조색2" xfId="38" builtinId="33" customBuiltin="1"/>
-    <cellStyle name="강조색3" xfId="42" builtinId="37" customBuiltin="1"/>
-    <cellStyle name="강조색4" xfId="46" builtinId="41" customBuiltin="1"/>
-    <cellStyle name="강조색5" xfId="50" builtinId="45" customBuiltin="1"/>
-    <cellStyle name="강조색6" xfId="54" builtinId="49" customBuiltin="1"/>
-    <cellStyle name="경고문" xfId="30" builtinId="11" customBuiltin="1"/>
-    <cellStyle name="계산" xfId="27" builtinId="22" customBuiltin="1"/>
-    <cellStyle name="나쁨" xfId="23" builtinId="27" customBuiltin="1"/>
-    <cellStyle name="메모" xfId="31" builtinId="10" customBuiltin="1"/>
-    <cellStyle name="백분율" xfId="16" builtinId="5"/>
-    <cellStyle name="보통" xfId="24" builtinId="28" customBuiltin="1"/>
-    <cellStyle name="설명 텍스트" xfId="32" builtinId="53" customBuiltin="1"/>
-    <cellStyle name="셀 확인" xfId="29" builtinId="23" customBuiltin="1"/>
-    <cellStyle name="쉼표" xfId="62" builtinId="3"/>
-    <cellStyle name="연결된 셀" xfId="28" builtinId="24" customBuiltin="1"/>
-    <cellStyle name="열어 본 하이퍼링크" xfId="11" builtinId="9" customBuiltin="1"/>
-    <cellStyle name="요약" xfId="33" builtinId="25" customBuiltin="1"/>
-    <cellStyle name="입력" xfId="25" builtinId="20" customBuiltin="1"/>
-    <cellStyle name="제목" xfId="17" builtinId="15" customBuiltin="1"/>
-    <cellStyle name="제목 1" xfId="18" builtinId="16" customBuiltin="1"/>
-    <cellStyle name="제목 2" xfId="19" builtinId="17" customBuiltin="1"/>
-    <cellStyle name="제목 3" xfId="20" builtinId="18" customBuiltin="1"/>
-    <cellStyle name="제목 4" xfId="21" builtinId="19" customBuiltin="1"/>
-    <cellStyle name="좋음" xfId="22" builtinId="26" customBuiltin="1"/>
-    <cellStyle name="출력" xfId="26" builtinId="21" customBuiltin="1"/>
-    <cellStyle name="표준" xfId="0" builtinId="0"/>
-    <cellStyle name="하이퍼링크" xfId="1" builtinId="8"/>
+    <cellStyle name="Total" xfId="33" builtinId="25" customBuiltin="1"/>
+    <cellStyle name="Warning Text" xfId="30" builtinId="11" customBuiltin="1"/>
   </cellStyles>
   <dxfs count="2">
     <dxf>
@@ -2007,17 +2010,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B59"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="132.25" customWidth="1"/>
+    <col min="2" max="2" width="132.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2">
       <c r="A3" s="1" t="s">
         <v>51</v>
       </c>
@@ -2025,232 +2028,232 @@
         <v>53</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2">
       <c r="B4" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2">
       <c r="B5" s="9">
         <v>2006</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2">
       <c r="B6" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2">
       <c r="B7" s="4" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2">
       <c r="B8" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2">
       <c r="B10" s="6" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2">
       <c r="B11" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:2">
       <c r="B12" s="9">
         <v>2016</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:2">
       <c r="B13" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:2">
       <c r="B14" s="4" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:2">
       <c r="B15" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="17" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:2">
       <c r="B17" s="6" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="18" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:2">
       <c r="B18" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="19" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:2">
       <c r="B19" s="9">
         <v>2015</v>
       </c>
     </row>
-    <row r="20" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:2">
       <c r="B20" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="21" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:2">
       <c r="B21" s="4" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="22" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:2">
       <c r="B22" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="24" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:2">
       <c r="B24" s="6" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="25" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:2">
       <c r="B25" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="26" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:2">
       <c r="B26" s="9">
         <v>2019</v>
       </c>
     </row>
-    <row r="27" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:2">
       <c r="B27" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="28" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:2">
       <c r="B28" s="4" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="30" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:2">
       <c r="B30" s="6" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="31" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:2">
       <c r="B31" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="32" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:2">
       <c r="B32" s="9">
         <v>2013</v>
       </c>
     </row>
-    <row r="33" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:2">
       <c r="B33" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="34" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:2">
       <c r="B34" s="4" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="35" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:2">
       <c r="B35" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="37" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:2">
       <c r="B37" s="6" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="38" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:2">
       <c r="B38" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="39" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:2">
       <c r="B39" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="40" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:2">
       <c r="B40" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="41" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:2">
       <c r="B41" s="19" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="42" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:2">
       <c r="B42" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="44" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="44" spans="2:2">
       <c r="B44" s="6" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="45" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="45" spans="2:2">
       <c r="B45" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="46" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="46" spans="2:2">
       <c r="B46" s="9">
         <v>2009</v>
       </c>
     </row>
-    <row r="47" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="47" spans="2:2">
       <c r="B47" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="48" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="48" spans="2:2">
       <c r="B48" s="19" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:2">
       <c r="B49" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:2">
       <c r="A51" s="1" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:2">
       <c r="A52" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:2">
       <c r="A54" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:2">
       <c r="A55" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:2">
       <c r="A57" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:2">
       <c r="A59" t="s">
         <v>99</v>
       </c>
@@ -2271,72 +2274,72 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:BB61"/>
-  <sheetFormatPr defaultColWidth="9.125" defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="19.375" customWidth="1"/>
-    <col min="2" max="27" width="7.75" customWidth="1"/>
-    <col min="28" max="28" width="7.125" customWidth="1"/>
+    <col min="1" max="1" width="19.42578125" customWidth="1"/>
+    <col min="2" max="27" width="7.7109375" customWidth="1"/>
+    <col min="28" max="28" width="7.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:54" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="81" t="s">
+    <row r="1" spans="1:54" ht="16.5" customHeight="1" thickBot="1">
+      <c r="A1" s="78" t="s">
         <v>64</v>
       </c>
-      <c r="B1" s="81"/>
-      <c r="C1" s="81"/>
-      <c r="D1" s="81"/>
-      <c r="E1" s="81"/>
-      <c r="F1" s="81"/>
-      <c r="G1" s="81"/>
-      <c r="H1" s="81"/>
-      <c r="I1" s="81"/>
-      <c r="J1" s="81"/>
-      <c r="K1" s="81"/>
-      <c r="L1" s="81"/>
-      <c r="M1" s="81"/>
-      <c r="N1" s="81"/>
-      <c r="O1" s="81"/>
-      <c r="P1" s="81"/>
-      <c r="Q1" s="81"/>
-      <c r="R1" s="81"/>
-      <c r="S1" s="81"/>
-      <c r="T1" s="81"/>
-      <c r="U1" s="81"/>
-      <c r="V1" s="81"/>
-      <c r="W1" s="81"/>
-      <c r="X1" s="81"/>
-      <c r="Y1" s="81"/>
-      <c r="Z1" s="81"/>
-      <c r="AA1" s="81"/>
-      <c r="AB1" s="81"/>
-      <c r="AC1" s="82"/>
-      <c r="AD1" s="82"/>
-      <c r="AE1" s="82"/>
-      <c r="AF1" s="82"/>
-      <c r="AG1" s="82"/>
-      <c r="AH1" s="82"/>
-      <c r="AI1" s="82"/>
-      <c r="AJ1" s="82"/>
-      <c r="AK1" s="82"/>
-      <c r="AL1" s="82"/>
-      <c r="AM1" s="82"/>
-      <c r="AN1" s="82"/>
-      <c r="AO1" s="82"/>
-      <c r="AP1" s="82"/>
-      <c r="AQ1" s="82"/>
-      <c r="AR1" s="82"/>
-      <c r="AS1" s="82"/>
-      <c r="AT1" s="82"/>
-      <c r="AU1" s="82"/>
-      <c r="AV1" s="82"/>
-      <c r="AW1" s="82"/>
-      <c r="AX1" s="82"/>
-      <c r="AY1" s="82"/>
-      <c r="AZ1" s="82"/>
-      <c r="BA1" s="82"/>
-      <c r="BB1" s="82"/>
-    </row>
-    <row r="2" spans="1:54" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B1" s="78"/>
+      <c r="C1" s="78"/>
+      <c r="D1" s="78"/>
+      <c r="E1" s="78"/>
+      <c r="F1" s="78"/>
+      <c r="G1" s="78"/>
+      <c r="H1" s="78"/>
+      <c r="I1" s="78"/>
+      <c r="J1" s="78"/>
+      <c r="K1" s="78"/>
+      <c r="L1" s="78"/>
+      <c r="M1" s="78"/>
+      <c r="N1" s="78"/>
+      <c r="O1" s="78"/>
+      <c r="P1" s="78"/>
+      <c r="Q1" s="78"/>
+      <c r="R1" s="78"/>
+      <c r="S1" s="78"/>
+      <c r="T1" s="78"/>
+      <c r="U1" s="78"/>
+      <c r="V1" s="78"/>
+      <c r="W1" s="78"/>
+      <c r="X1" s="78"/>
+      <c r="Y1" s="78"/>
+      <c r="Z1" s="78"/>
+      <c r="AA1" s="78"/>
+      <c r="AB1" s="78"/>
+      <c r="AC1" s="79"/>
+      <c r="AD1" s="79"/>
+      <c r="AE1" s="79"/>
+      <c r="AF1" s="79"/>
+      <c r="AG1" s="79"/>
+      <c r="AH1" s="79"/>
+      <c r="AI1" s="79"/>
+      <c r="AJ1" s="79"/>
+      <c r="AK1" s="79"/>
+      <c r="AL1" s="79"/>
+      <c r="AM1" s="79"/>
+      <c r="AN1" s="79"/>
+      <c r="AO1" s="79"/>
+      <c r="AP1" s="79"/>
+      <c r="AQ1" s="79"/>
+      <c r="AR1" s="79"/>
+      <c r="AS1" s="79"/>
+      <c r="AT1" s="79"/>
+      <c r="AU1" s="79"/>
+      <c r="AV1" s="79"/>
+      <c r="AW1" s="79"/>
+      <c r="AX1" s="79"/>
+      <c r="AY1" s="79"/>
+      <c r="AZ1" s="79"/>
+      <c r="BA1" s="79"/>
+      <c r="BB1" s="79"/>
+    </row>
+    <row r="2" spans="1:54" ht="16.5" customHeight="1">
       <c r="A2" s="38"/>
       <c r="B2" s="39">
         <v>1980</v>
@@ -2446,7 +2449,7 @@
       <c r="BA2" s="45"/>
       <c r="BB2" s="46"/>
     </row>
-    <row r="3" spans="1:54" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:54" ht="16.5" customHeight="1">
       <c r="A3" s="47" t="s">
         <v>65</v>
       </c>
@@ -2558,7 +2561,7 @@
       <c r="BA3" s="48"/>
       <c r="BB3" s="48"/>
     </row>
-    <row r="4" spans="1:54" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:54" ht="16.5" customHeight="1">
       <c r="A4" s="50" t="s">
         <v>67</v>
       </c>
@@ -2670,7 +2673,7 @@
       <c r="BA4" s="52"/>
       <c r="BB4" s="52"/>
     </row>
-    <row r="5" spans="1:54" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:54" ht="16.5" customHeight="1">
       <c r="A5" s="50" t="s">
         <v>68</v>
       </c>
@@ -2782,7 +2785,7 @@
       <c r="BA5" s="52"/>
       <c r="BB5" s="52"/>
     </row>
-    <row r="6" spans="1:54" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:54" ht="16.5" customHeight="1">
       <c r="A6" s="50" t="s">
         <v>69</v>
       </c>
@@ -2894,7 +2897,7 @@
       <c r="BA6" s="52"/>
       <c r="BB6" s="52"/>
     </row>
-    <row r="7" spans="1:54" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:54" ht="16.5" customHeight="1">
       <c r="A7" s="50" t="s">
         <v>70</v>
       </c>
@@ -3006,7 +3009,7 @@
       <c r="BA7" s="52"/>
       <c r="BB7" s="52"/>
     </row>
-    <row r="8" spans="1:54" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:54" ht="16.5" customHeight="1">
       <c r="A8" s="50" t="s">
         <v>71</v>
       </c>
@@ -3118,7 +3121,7 @@
       <c r="BA8" s="52"/>
       <c r="BB8" s="52"/>
     </row>
-    <row r="9" spans="1:54" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:54" ht="16.5" customHeight="1">
       <c r="A9" s="53" t="s">
         <v>72</v>
       </c>
@@ -3176,7 +3179,7 @@
       <c r="BA9" s="54"/>
       <c r="BB9" s="54"/>
     </row>
-    <row r="10" spans="1:54" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:54" ht="16.5" customHeight="1">
       <c r="A10" s="50" t="s">
         <v>67</v>
       </c>
@@ -3290,7 +3293,7 @@
       <c r="BA10" s="56"/>
       <c r="BB10" s="56"/>
     </row>
-    <row r="11" spans="1:54" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:54" ht="16.5" customHeight="1">
       <c r="A11" s="50" t="s">
         <v>68</v>
       </c>
@@ -3402,7 +3405,7 @@
       <c r="BA11" s="56"/>
       <c r="BB11" s="56"/>
     </row>
-    <row r="12" spans="1:54" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:54" ht="16.5" customHeight="1">
       <c r="A12" s="50" t="s">
         <v>69</v>
       </c>
@@ -3514,7 +3517,7 @@
       <c r="BA12" s="56"/>
       <c r="BB12" s="56"/>
     </row>
-    <row r="13" spans="1:54" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:54" ht="16.5" customHeight="1">
       <c r="A13" s="50" t="s">
         <v>70</v>
       </c>
@@ -3626,7 +3629,7 @@
       <c r="BA13" s="56"/>
       <c r="BB13" s="56"/>
     </row>
-    <row r="14" spans="1:54" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:54" ht="16.5" customHeight="1">
       <c r="A14" s="50" t="s">
         <v>71</v>
       </c>
@@ -3738,7 +3741,7 @@
       <c r="BA14" s="56"/>
       <c r="BB14" s="56"/>
     </row>
-    <row r="15" spans="1:54" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:54" ht="16.5" customHeight="1">
       <c r="A15" s="47" t="s">
         <v>73</v>
       </c>
@@ -3796,7 +3799,7 @@
       <c r="BA15" s="58"/>
       <c r="BB15" s="58"/>
     </row>
-    <row r="16" spans="1:54" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:54" ht="16.5" customHeight="1">
       <c r="A16" s="50" t="s">
         <v>67</v>
       </c>
@@ -3908,7 +3911,7 @@
       <c r="BA16" s="59"/>
       <c r="BB16" s="59"/>
     </row>
-    <row r="17" spans="1:54" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:54" ht="16.5" customHeight="1">
       <c r="A17" s="50" t="s">
         <v>68</v>
       </c>
@@ -4020,7 +4023,7 @@
       <c r="BA17" s="59"/>
       <c r="BB17" s="59"/>
     </row>
-    <row r="18" spans="1:54" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:54" ht="16.5" customHeight="1">
       <c r="A18" s="50" t="s">
         <v>69</v>
       </c>
@@ -4132,7 +4135,7 @@
       <c r="BA18" s="59"/>
       <c r="BB18" s="59"/>
     </row>
-    <row r="19" spans="1:54" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:54" ht="16.5" customHeight="1">
       <c r="A19" s="50" t="s">
         <v>70</v>
       </c>
@@ -4244,7 +4247,7 @@
       <c r="BA19" s="59"/>
       <c r="BB19" s="59"/>
     </row>
-    <row r="20" spans="1:54" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:54" ht="16.5" customHeight="1" thickBot="1">
       <c r="A20" s="60" t="s">
         <v>71</v>
       </c>
@@ -4356,68 +4359,68 @@
       <c r="BA20" s="59"/>
       <c r="BB20" s="59"/>
     </row>
-    <row r="21" spans="1:54" s="63" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="83" t="s">
+    <row r="21" spans="1:54" s="63" customFormat="1" ht="12.75" customHeight="1">
+      <c r="A21" s="80" t="s">
         <v>74</v>
       </c>
-      <c r="B21" s="83"/>
-      <c r="C21" s="83"/>
-      <c r="D21" s="83"/>
-      <c r="E21" s="83"/>
-      <c r="F21" s="83"/>
-      <c r="G21" s="83"/>
-      <c r="H21" s="83"/>
-      <c r="I21" s="83"/>
-      <c r="J21" s="83"/>
-      <c r="K21" s="83"/>
-      <c r="L21" s="83"/>
-      <c r="M21" s="83"/>
-      <c r="N21" s="83"/>
-      <c r="O21" s="83"/>
-      <c r="P21" s="83"/>
-      <c r="Q21" s="83"/>
-    </row>
-    <row r="22" spans="1:54" s="63" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="84"/>
-      <c r="B22" s="84"/>
-      <c r="C22" s="84"/>
-      <c r="D22" s="84"/>
-      <c r="E22" s="84"/>
-      <c r="F22" s="84"/>
-      <c r="G22" s="84"/>
-      <c r="H22" s="84"/>
-      <c r="I22" s="84"/>
-      <c r="J22" s="84"/>
-      <c r="K22" s="84"/>
-      <c r="L22" s="84"/>
-      <c r="M22" s="84"/>
-      <c r="N22" s="84"/>
-      <c r="O22" s="84"/>
-      <c r="P22" s="84"/>
-      <c r="Q22" s="84"/>
-    </row>
-    <row r="23" spans="1:54" s="63" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="84" t="s">
+      <c r="B21" s="80"/>
+      <c r="C21" s="80"/>
+      <c r="D21" s="80"/>
+      <c r="E21" s="80"/>
+      <c r="F21" s="80"/>
+      <c r="G21" s="80"/>
+      <c r="H21" s="80"/>
+      <c r="I21" s="80"/>
+      <c r="J21" s="80"/>
+      <c r="K21" s="80"/>
+      <c r="L21" s="80"/>
+      <c r="M21" s="80"/>
+      <c r="N21" s="80"/>
+      <c r="O21" s="80"/>
+      <c r="P21" s="80"/>
+      <c r="Q21" s="80"/>
+    </row>
+    <row r="22" spans="1:54" s="63" customFormat="1" ht="12.75" customHeight="1">
+      <c r="A22" s="81"/>
+      <c r="B22" s="81"/>
+      <c r="C22" s="81"/>
+      <c r="D22" s="81"/>
+      <c r="E22" s="81"/>
+      <c r="F22" s="81"/>
+      <c r="G22" s="81"/>
+      <c r="H22" s="81"/>
+      <c r="I22" s="81"/>
+      <c r="J22" s="81"/>
+      <c r="K22" s="81"/>
+      <c r="L22" s="81"/>
+      <c r="M22" s="81"/>
+      <c r="N22" s="81"/>
+      <c r="O22" s="81"/>
+      <c r="P22" s="81"/>
+      <c r="Q22" s="81"/>
+    </row>
+    <row r="23" spans="1:54" s="63" customFormat="1" ht="12.75" customHeight="1">
+      <c r="A23" s="81" t="s">
         <v>75</v>
       </c>
-      <c r="B23" s="84"/>
-      <c r="C23" s="84"/>
-      <c r="D23" s="84"/>
-      <c r="E23" s="84"/>
-      <c r="F23" s="84"/>
-      <c r="G23" s="84"/>
-      <c r="H23" s="84"/>
-      <c r="I23" s="84"/>
-      <c r="J23" s="84"/>
-      <c r="K23" s="84"/>
-      <c r="L23" s="84"/>
-      <c r="M23" s="84"/>
-      <c r="N23" s="84"/>
-      <c r="O23" s="84"/>
-      <c r="P23" s="84"/>
-      <c r="Q23" s="84"/>
-    </row>
-    <row r="24" spans="1:54" s="63" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B23" s="81"/>
+      <c r="C23" s="81"/>
+      <c r="D23" s="81"/>
+      <c r="E23" s="81"/>
+      <c r="F23" s="81"/>
+      <c r="G23" s="81"/>
+      <c r="H23" s="81"/>
+      <c r="I23" s="81"/>
+      <c r="J23" s="81"/>
+      <c r="K23" s="81"/>
+      <c r="L23" s="81"/>
+      <c r="M23" s="81"/>
+      <c r="N23" s="81"/>
+      <c r="O23" s="81"/>
+      <c r="P23" s="81"/>
+      <c r="Q23" s="81"/>
+    </row>
+    <row r="24" spans="1:54" s="63" customFormat="1" ht="12.75" customHeight="1">
       <c r="A24" s="77" t="s">
         <v>76</v>
       </c>
@@ -4438,7 +4441,7 @@
       <c r="P24" s="77"/>
       <c r="Q24" s="77"/>
     </row>
-    <row r="25" spans="1:54" s="63" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:54" s="63" customFormat="1" ht="12.75" customHeight="1">
       <c r="A25" s="77" t="s">
         <v>77</v>
       </c>
@@ -4459,130 +4462,130 @@
       <c r="P25" s="77"/>
       <c r="Q25" s="77"/>
     </row>
-    <row r="26" spans="1:54" s="63" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="78" t="s">
+    <row r="26" spans="1:54" s="63" customFormat="1" ht="27.75" customHeight="1">
+      <c r="A26" s="82" t="s">
         <v>78</v>
       </c>
-      <c r="B26" s="78"/>
-      <c r="C26" s="78"/>
-      <c r="D26" s="78"/>
-      <c r="E26" s="78"/>
-      <c r="F26" s="78"/>
-      <c r="G26" s="78"/>
-      <c r="H26" s="78"/>
-      <c r="I26" s="78"/>
-      <c r="J26" s="78"/>
-      <c r="K26" s="78"/>
-      <c r="L26" s="78"/>
-      <c r="M26" s="78"/>
-      <c r="N26" s="78"/>
-      <c r="O26" s="78"/>
-      <c r="P26" s="78"/>
-      <c r="Q26" s="78"/>
-    </row>
-    <row r="27" spans="1:54" s="63" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="78"/>
-      <c r="B27" s="78"/>
-      <c r="C27" s="78"/>
-      <c r="D27" s="78"/>
-      <c r="E27" s="78"/>
-      <c r="F27" s="78"/>
-      <c r="G27" s="78"/>
-      <c r="H27" s="78"/>
-      <c r="I27" s="78"/>
-      <c r="J27" s="78"/>
-      <c r="K27" s="78"/>
-      <c r="L27" s="78"/>
-      <c r="M27" s="78"/>
-      <c r="N27" s="78"/>
-      <c r="O27" s="78"/>
-      <c r="P27" s="78"/>
-      <c r="Q27" s="78"/>
-    </row>
-    <row r="28" spans="1:54" s="63" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="79" t="s">
+      <c r="B26" s="82"/>
+      <c r="C26" s="82"/>
+      <c r="D26" s="82"/>
+      <c r="E26" s="82"/>
+      <c r="F26" s="82"/>
+      <c r="G26" s="82"/>
+      <c r="H26" s="82"/>
+      <c r="I26" s="82"/>
+      <c r="J26" s="82"/>
+      <c r="K26" s="82"/>
+      <c r="L26" s="82"/>
+      <c r="M26" s="82"/>
+      <c r="N26" s="82"/>
+      <c r="O26" s="82"/>
+      <c r="P26" s="82"/>
+      <c r="Q26" s="82"/>
+    </row>
+    <row r="27" spans="1:54" s="63" customFormat="1" ht="12.75" customHeight="1">
+      <c r="A27" s="82"/>
+      <c r="B27" s="82"/>
+      <c r="C27" s="82"/>
+      <c r="D27" s="82"/>
+      <c r="E27" s="82"/>
+      <c r="F27" s="82"/>
+      <c r="G27" s="82"/>
+      <c r="H27" s="82"/>
+      <c r="I27" s="82"/>
+      <c r="J27" s="82"/>
+      <c r="K27" s="82"/>
+      <c r="L27" s="82"/>
+      <c r="M27" s="82"/>
+      <c r="N27" s="82"/>
+      <c r="O27" s="82"/>
+      <c r="P27" s="82"/>
+      <c r="Q27" s="82"/>
+    </row>
+    <row r="28" spans="1:54" s="63" customFormat="1" ht="12.75" customHeight="1">
+      <c r="A28" s="83" t="s">
         <v>79</v>
       </c>
-      <c r="B28" s="79"/>
-      <c r="C28" s="79"/>
-      <c r="D28" s="79"/>
-      <c r="E28" s="79"/>
-      <c r="F28" s="79"/>
-      <c r="G28" s="79"/>
-      <c r="H28" s="79"/>
-      <c r="I28" s="79"/>
-      <c r="J28" s="79"/>
-      <c r="K28" s="79"/>
-      <c r="L28" s="79"/>
-      <c r="M28" s="79"/>
-      <c r="N28" s="79"/>
-      <c r="O28" s="79"/>
-      <c r="P28" s="79"/>
-      <c r="Q28" s="79"/>
-    </row>
-    <row r="29" spans="1:54" s="63" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="80" t="s">
+      <c r="B28" s="83"/>
+      <c r="C28" s="83"/>
+      <c r="D28" s="83"/>
+      <c r="E28" s="83"/>
+      <c r="F28" s="83"/>
+      <c r="G28" s="83"/>
+      <c r="H28" s="83"/>
+      <c r="I28" s="83"/>
+      <c r="J28" s="83"/>
+      <c r="K28" s="83"/>
+      <c r="L28" s="83"/>
+      <c r="M28" s="83"/>
+      <c r="N28" s="83"/>
+      <c r="O28" s="83"/>
+      <c r="P28" s="83"/>
+      <c r="Q28" s="83"/>
+    </row>
+    <row r="29" spans="1:54" s="63" customFormat="1" ht="25.5" customHeight="1">
+      <c r="A29" s="84" t="s">
         <v>80</v>
       </c>
-      <c r="B29" s="80"/>
-      <c r="C29" s="80"/>
-      <c r="D29" s="80"/>
-      <c r="E29" s="80"/>
-      <c r="F29" s="80"/>
-      <c r="G29" s="80"/>
-      <c r="H29" s="80"/>
-      <c r="I29" s="80"/>
-      <c r="J29" s="80"/>
-      <c r="K29" s="80"/>
-      <c r="L29" s="80"/>
-      <c r="M29" s="80"/>
-      <c r="N29" s="80"/>
-      <c r="O29" s="80"/>
-      <c r="P29" s="80"/>
-      <c r="Q29" s="80"/>
-    </row>
-    <row r="33" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="34" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="35" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="36" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="37" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="38" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="39" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="40" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="41" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="42" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="43" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="44" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="45" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="46" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="47" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="48" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="49" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="50" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="51" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="52" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="53" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="54" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="55" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="56" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="57" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="58" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="59" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="60" customFormat="1" x14ac:dyDescent="0.3"/>
-    <row r="61" customFormat="1" x14ac:dyDescent="0.3"/>
+      <c r="B29" s="84"/>
+      <c r="C29" s="84"/>
+      <c r="D29" s="84"/>
+      <c r="E29" s="84"/>
+      <c r="F29" s="84"/>
+      <c r="G29" s="84"/>
+      <c r="H29" s="84"/>
+      <c r="I29" s="84"/>
+      <c r="J29" s="84"/>
+      <c r="K29" s="84"/>
+      <c r="L29" s="84"/>
+      <c r="M29" s="84"/>
+      <c r="N29" s="84"/>
+      <c r="O29" s="84"/>
+      <c r="P29" s="84"/>
+      <c r="Q29" s="84"/>
+    </row>
+    <row r="33" customFormat="1"/>
+    <row r="34" customFormat="1"/>
+    <row r="35" customFormat="1"/>
+    <row r="36" customFormat="1"/>
+    <row r="37" customFormat="1"/>
+    <row r="38" customFormat="1"/>
+    <row r="39" customFormat="1"/>
+    <row r="40" customFormat="1"/>
+    <row r="41" customFormat="1"/>
+    <row r="42" customFormat="1"/>
+    <row r="43" customFormat="1"/>
+    <row r="44" customFormat="1"/>
+    <row r="45" customFormat="1"/>
+    <row r="46" customFormat="1"/>
+    <row r="47" customFormat="1"/>
+    <row r="48" customFormat="1"/>
+    <row r="49" customFormat="1"/>
+    <row r="50" customFormat="1"/>
+    <row r="51" customFormat="1"/>
+    <row r="52" customFormat="1"/>
+    <row r="53" customFormat="1"/>
+    <row r="54" customFormat="1"/>
+    <row r="55" customFormat="1"/>
+    <row r="56" customFormat="1"/>
+    <row r="57" customFormat="1"/>
+    <row r="58" customFormat="1"/>
+    <row r="59" customFormat="1"/>
+    <row r="60" customFormat="1"/>
+    <row r="61" customFormat="1"/>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="A25:Q25"/>
+    <mergeCell ref="A26:Q26"/>
+    <mergeCell ref="A27:Q27"/>
+    <mergeCell ref="A28:Q28"/>
+    <mergeCell ref="A29:Q29"/>
     <mergeCell ref="A24:Q24"/>
     <mergeCell ref="A1:AB1"/>
     <mergeCell ref="AC1:BB1"/>
     <mergeCell ref="A21:Q21"/>
     <mergeCell ref="A22:Q22"/>
     <mergeCell ref="A23:Q23"/>
-    <mergeCell ref="A25:Q25"/>
-    <mergeCell ref="A26:Q26"/>
-    <mergeCell ref="A27:Q27"/>
-    <mergeCell ref="A28:Q28"/>
-    <mergeCell ref="A29:Q29"/>
   </mergeCells>
   <phoneticPr fontId="38" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4592,17 +4595,17 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:E48"/>
-  <sheetFormatPr defaultColWidth="9.125" defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="30.125" style="3" customWidth="1"/>
-    <col min="2" max="2" width="29.875" style="3" customWidth="1"/>
-    <col min="3" max="3" width="25.25" style="3" customWidth="1"/>
-    <col min="4" max="4" width="22.75" style="3" customWidth="1"/>
-    <col min="5" max="5" width="25.125" style="3" customWidth="1"/>
-    <col min="6" max="16384" width="9.125" style="3"/>
+    <col min="1" max="1" width="30.140625" style="3" customWidth="1"/>
+    <col min="2" max="2" width="29.85546875" style="3" customWidth="1"/>
+    <col min="3" max="3" width="25.28515625" style="3" customWidth="1"/>
+    <col min="4" max="4" width="22.7109375" style="3" customWidth="1"/>
+    <col min="5" max="5" width="25.140625" style="3" customWidth="1"/>
+    <col min="6" max="16384" width="9.140625" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" customFormat="1" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" customFormat="1" ht="15.75" thickBot="1">
       <c r="A1" s="6" t="s">
         <v>52</v>
       </c>
@@ -4611,7 +4614,7 @@
       <c r="D1" s="33"/>
       <c r="E1" s="33"/>
     </row>
-    <row r="2" spans="1:5" s="2" customFormat="1" ht="66" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" s="2" customFormat="1" ht="60">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -4628,7 +4631,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" ht="15.75" thickBot="1">
       <c r="A3" s="3">
         <v>13</v>
       </c>
@@ -4648,12 +4651,12 @@
         <v>13.378781688359696</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" ht="15.75" thickBot="1">
       <c r="A5" s="10" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="33" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" ht="30">
       <c r="A6" s="7" t="s">
         <v>59</v>
       </c>
@@ -4668,7 +4671,7 @@
       </c>
       <c r="E6" s="2"/>
     </row>
-    <row r="7" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" ht="15.75" thickBot="1">
       <c r="A7" s="68">
         <v>28</v>
       </c>
@@ -4683,7 +4686,7 @@
       </c>
       <c r="E7" s="67"/>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:5">
       <c r="A10" s="10" t="s">
         <v>56</v>
       </c>
@@ -4692,14 +4695,14 @@
       <c r="D10" s="34"/>
       <c r="E10" s="34"/>
     </row>
-    <row r="11" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:5" s="9" customFormat="1">
       <c r="A11" s="15" t="s">
         <v>33</v>
       </c>
       <c r="B11" s="14"/>
       <c r="C11" s="15"/>
     </row>
-    <row r="12" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:5" s="9" customFormat="1">
       <c r="A12" s="9" t="s">
         <v>34</v>
       </c>
@@ -4707,7 +4710,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="13" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:5" s="9" customFormat="1">
       <c r="A13" s="9" t="s">
         <v>36</v>
       </c>
@@ -4715,7 +4718,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="14" spans="1:5" s="9" customFormat="1" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" s="9" customFormat="1" ht="15.75" thickBot="1">
       <c r="A14" s="9" t="s">
         <v>38</v>
       </c>
@@ -4723,17 +4726,17 @@
         <v>39</v>
       </c>
     </row>
-    <row r="15" spans="1:5" s="9" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:5" s="9" customFormat="1">
       <c r="A15" s="17" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="16" spans="1:5" s="9" customFormat="1" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:5" s="9" customFormat="1" ht="15.75" thickBot="1">
       <c r="A16" s="18">
         <v>24</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:5">
       <c r="A18" s="10" t="s">
         <v>21</v>
       </c>
@@ -4742,7 +4745,7 @@
       <c r="D18" s="34"/>
       <c r="E18" s="34"/>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:5">
       <c r="A19" s="15" t="s">
         <v>10</v>
       </c>
@@ -4753,7 +4756,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:5">
       <c r="A20" t="s">
         <v>22</v>
       </c>
@@ -4764,7 +4767,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="21" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:5" ht="15.75" thickBot="1">
       <c r="A21" t="s">
         <v>24</v>
       </c>
@@ -4775,7 +4778,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="22" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:5" ht="15.75" thickBot="1">
       <c r="A22"/>
       <c r="B22" s="11" t="s">
         <v>26</v>
@@ -4784,17 +4787,17 @@
         <v>34</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:5">
       <c r="A23" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:5">
       <c r="A24" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:5">
       <c r="A26" s="10" t="s">
         <v>13</v>
       </c>
@@ -4803,7 +4806,7 @@
       <c r="D26" s="34"/>
       <c r="E26" s="34"/>
     </row>
-    <row r="27" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:5" ht="15.75" thickBot="1">
       <c r="A27" s="15" t="s">
         <v>10</v>
       </c>
@@ -4814,7 +4817,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="28" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:5" ht="15.75" thickBot="1">
       <c r="A28" t="s">
         <v>14</v>
       </c>
@@ -4825,7 +4828,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="30" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:5" ht="15.75" thickBot="1">
       <c r="A30" s="10" t="s">
         <v>58</v>
       </c>
@@ -4834,7 +4837,7 @@
       <c r="D30" s="34"/>
       <c r="E30" s="34"/>
     </row>
-    <row r="31" spans="1:5" ht="33" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:5" ht="30">
       <c r="A31" s="21" t="s">
         <v>43</v>
       </c>
@@ -4851,7 +4854,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:5">
       <c r="A32" s="20">
         <v>1997</v>
       </c>
@@ -4864,7 +4867,7 @@
       <c r="D32" s="9"/>
       <c r="E32" s="9"/>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:5">
       <c r="A33" s="20">
         <v>1998</v>
       </c>
@@ -4883,7 +4886,7 @@
         <v>6.6484424338501588E-2</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:5">
       <c r="A34" s="20">
         <v>1999</v>
       </c>
@@ -4902,7 +4905,7 @@
         <v>2.9143636995467476E-2</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:5">
       <c r="A35" s="20">
         <v>2000</v>
       </c>
@@ -4921,7 +4924,7 @@
         <v>6.8191523924614153E-2</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:5">
       <c r="A36" s="20">
         <v>2001</v>
       </c>
@@ -4940,7 +4943,7 @@
         <v>4.0815360868813244E-3</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:5">
       <c r="A37" s="20">
         <v>2002</v>
       </c>
@@ -4959,7 +4962,7 @@
         <v>0.10769048766665149</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:5">
       <c r="A38" s="20">
         <v>2003</v>
       </c>
@@ -4978,7 +4981,7 @@
         <v>5.9053805049687755E-2</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:5">
       <c r="A39" s="20">
         <v>2004</v>
       </c>
@@ -4997,7 +5000,7 @@
         <v>5.8670234757052138E-2</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:5">
       <c r="A40" s="20">
         <v>2005</v>
       </c>
@@ -5016,7 +5019,7 @@
         <v>6.1781753631599455E-2</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:5">
       <c r="A41" s="20">
         <v>2006</v>
       </c>
@@ -5035,7 +5038,7 @@
         <v>6.5906687839630079E-2</v>
       </c>
     </row>
-    <row r="42" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:5" ht="15.75" thickBot="1">
       <c r="A42" s="25">
         <v>2007</v>
       </c>
@@ -5054,14 +5057,14 @@
         <v>5.9604038733197397E-2</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:5">
       <c r="A43"/>
       <c r="B43"/>
       <c r="C43"/>
       <c r="D43"/>
       <c r="E43"/>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:5">
       <c r="A44" s="1" t="s">
         <v>47</v>
       </c>
@@ -5069,7 +5072,7 @@
       <c r="C44"/>
       <c r="D44"/>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:5">
       <c r="A45" s="28">
         <f>AVERAGE(E33:E42)</f>
         <v>5.8060812902328285E-2</v>
@@ -5078,13 +5081,13 @@
       <c r="C45"/>
       <c r="D45"/>
     </row>
-    <row r="46" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:5" ht="15.75" thickBot="1">
       <c r="A46"/>
       <c r="B46"/>
       <c r="C46"/>
       <c r="D46"/>
     </row>
-    <row r="47" spans="1:5" ht="33" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:5" ht="30">
       <c r="A47" s="36" t="s">
         <v>48</v>
       </c>
@@ -5092,7 +5095,7 @@
       <c r="C47"/>
       <c r="D47"/>
     </row>
-    <row r="48" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:5" ht="15.75" thickBot="1">
       <c r="A48" s="35">
         <f>1/A45</f>
         <v>17.22332068760786</v>
@@ -5112,25 +5115,25 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD149825-14BA-415D-91AD-354F00EEF420}">
-  <dimension ref="A1:K40"/>
-  <sheetFormatPr defaultColWidth="8.75" defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:K43"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="19.125" style="70" customWidth="1"/>
-    <col min="2" max="2" width="11.125" style="70" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="10.125" style="70" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="12.5" style="70" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.125" style="70" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.5" style="70" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.125" style="70" bestFit="1" customWidth="1"/>
-    <col min="10" max="16384" width="8.75" style="70"/>
+    <col min="1" max="1" width="19.140625" style="70" customWidth="1"/>
+    <col min="2" max="2" width="11.140625" style="70" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="10.140625" style="70" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="12.42578125" style="70" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.140625" style="70" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.42578125" style="70" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.140625" style="70" bestFit="1" customWidth="1"/>
+    <col min="10" max="16384" width="8.7109375" style="70"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9">
       <c r="A1" s="70" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9">
       <c r="B2" s="70" t="s">
         <v>101</v>
       </c>
@@ -5156,7 +5159,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9">
       <c r="B3" s="70" t="s">
         <v>52</v>
       </c>
@@ -5182,7 +5185,7 @@
         <v>7728.5710293009906</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9">
       <c r="B4" s="70" t="s">
         <v>55</v>
       </c>
@@ -5208,7 +5211,7 @@
         <v>3161.4504274369956</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9">
       <c r="B5" s="70" t="s">
         <v>56</v>
       </c>
@@ -5234,7 +5237,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9">
       <c r="B6" s="70" t="s">
         <v>21</v>
       </c>
@@ -5260,7 +5263,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9">
       <c r="B7" s="70" t="s">
         <v>13</v>
       </c>
@@ -5286,7 +5289,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9">
       <c r="B8" s="70" t="s">
         <v>58</v>
       </c>
@@ -5312,12 +5315,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9">
       <c r="A10" s="70" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9">
       <c r="B11" s="70" t="s">
         <v>101</v>
       </c>
@@ -5343,7 +5346,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:9">
       <c r="B12" s="70" t="s">
         <v>52</v>
       </c>
@@ -5369,7 +5372,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:9">
       <c r="B13" s="70" t="s">
         <v>55</v>
       </c>
@@ -5395,7 +5398,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:9">
       <c r="B14" s="70" t="s">
         <v>56</v>
       </c>
@@ -5421,7 +5424,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:9">
       <c r="B15" s="70" t="s">
         <v>21</v>
       </c>
@@ -5447,7 +5450,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:9">
       <c r="B16" s="70" t="s">
         <v>13</v>
       </c>
@@ -5473,7 +5476,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:9">
       <c r="B17" s="70" t="s">
         <v>58</v>
       </c>
@@ -5499,12 +5502,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:9">
       <c r="A20" s="70" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:9">
       <c r="B22" s="70">
         <v>2019</v>
       </c>
@@ -5512,7 +5515,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:9">
       <c r="A23" s="70" t="s">
         <v>111</v>
       </c>
@@ -5528,7 +5531,7 @@
         <v>11.724644713881862</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:9">
       <c r="A24" s="70" t="s">
         <v>112</v>
       </c>
@@ -5544,7 +5547,7 @@
         <v>11.325209578137313</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:9">
       <c r="A25" s="70" t="s">
         <v>113</v>
       </c>
@@ -5556,7 +5559,7 @@
         <v>0.27844474080318277</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:9">
       <c r="A26" s="70" t="s">
         <v>114</v>
       </c>
@@ -5568,13 +5571,13 @@
         <v>0.38904941180819808</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:9">
       <c r="C27" s="72"/>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:9">
       <c r="C28" s="72"/>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:9">
       <c r="A29" s="70" t="s">
         <v>115</v>
       </c>
@@ -5590,7 +5593,7 @@
         <v>20.43541033331925</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:9">
       <c r="A30" s="70" t="s">
         <v>116</v>
       </c>
@@ -5606,7 +5609,7 @@
         <v>13.907940419258974</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:9">
       <c r="A31" s="70" t="s">
         <v>117</v>
       </c>
@@ -5618,7 +5621,7 @@
         <v>6.8718275287445466E-2</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:9">
       <c r="A32" s="70" t="s">
         <v>118</v>
       </c>
@@ -5630,7 +5633,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:11">
       <c r="A34" s="74" t="s">
         <v>128</v>
       </c>
@@ -5641,7 +5644,7 @@
       <c r="F34" s="74"/>
       <c r="G34" s="74"/>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:11">
       <c r="A35" s="74"/>
       <c r="B35" s="74">
         <v>2000</v>
@@ -5664,7 +5667,7 @@
       <c r="J35" s="3"/>
       <c r="K35" s="3"/>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:11">
       <c r="A36" s="74" t="s">
         <v>121</v>
       </c>
@@ -5694,7 +5697,7 @@
       </c>
       <c r="J36" s="75"/>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:11">
       <c r="A37" s="74" t="s">
         <v>122</v>
       </c>
@@ -5724,7 +5727,7 @@
       </c>
       <c r="J37" s="75"/>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:11">
       <c r="A38" s="74" t="s">
         <v>123</v>
       </c>
@@ -5753,7 +5756,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:11">
       <c r="A39" s="74" t="s">
         <v>124</v>
       </c>
@@ -5782,7 +5785,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:11">
       <c r="A40" s="74" t="s">
         <v>125</v>
       </c>
@@ -5803,6 +5806,11 @@
       </c>
       <c r="G40" s="76">
         <v>16</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11">
+      <c r="A43" s="70" t="s">
+        <v>132</v>
       </c>
     </row>
   </sheetData>
@@ -5818,14 +5826,14 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="14.625" customWidth="1"/>
+    <col min="1" max="1" width="14.5703125" customWidth="1"/>
     <col min="2" max="2" width="19" customWidth="1"/>
-    <col min="3" max="3" width="15.625" customWidth="1"/>
+    <col min="3" max="3" width="15.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="33" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="45">
       <c r="A1" s="69" t="s">
         <v>100</v>
       </c>
@@ -5836,20 +5844,19 @@
         <v>93</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>52</v>
       </c>
       <c r="B2" s="73">
-        <f>'SK calcs'!G36</f>
-        <v>15.6</v>
+        <v>13</v>
       </c>
       <c r="C2" s="73">
         <f>AVERAGE('SK calcs'!$G$38:$G$39)</f>
         <v>17.75</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>55</v>
       </c>
@@ -5862,7 +5869,7 @@
         <v>17.75</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>56</v>
       </c>
@@ -5871,11 +5878,11 @@
         <v>24</v>
       </c>
       <c r="C4" s="37">
-        <f t="shared" ref="C2:C7" si="0">B4</f>
+        <f t="shared" ref="C4:C7" si="0">B4</f>
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
         <v>21</v>
       </c>
@@ -5888,7 +5895,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
         <v>13</v>
       </c>
@@ -5901,7 +5908,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3">
       <c r="A7" t="s">
         <v>58</v>
       </c>
@@ -5921,6 +5928,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100E59C87379D9A4242BB3A95F198D6F941" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="07a235b40ffe2d9a960bde50f6511605">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="40f4d404-d193-41dc-bb72-733c1e774208" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="485fc8e6f691b86ce0aee9b7e82feca0" ns2:_="">
     <xsd:import namespace="40f4d404-d193-41dc-bb72-733c1e774208"/>
@@ -6064,15 +6080,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement/>
@@ -6080,6 +6087,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{48C589ED-403D-43C7-8D67-619C9CBC31EC}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{26A9F799-6530-441C-9A49-116D487C0166}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -6093,14 +6108,6 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{48C589ED-403D-43C7-8D67-619C9CBC31EC}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>